<commit_message>
Add Horse Stance Hold through mobility routes
Agent: horsehold
</commit_message>
<xml_diff>
--- a/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
+++ b/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="R223e84657cf44f7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Rd1b544c9eb764f14"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9122,6 +9122,32 @@
         <x:v>Don't round the spine.</x:v>
       </x:c>
     </x:row>
+    <x:row r="217" ht="90" customHeight="1">
+      <x:c r="A217" s="5" t="str">
+        <x:v>Mobility</x:v>
+      </x:c>
+      <x:c r="B217" s="5" t="str">
+        <x:v>Horse Stance Hold</x:v>
+      </x:c>
+      <x:c r="C217" s="5" t="str">
+        <x:v>Groin, Quads, Glutes</x:v>
+      </x:c>
+      <x:c r="D217" s="5" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E217" s="5" t="str">
+        <x:v>everyone</x:v>
+      </x:c>
+      <x:c r="F217" s="5" t="str">
+        <x:v>2 × 60-second total holds. Bodyweight; use a higher or narrower stance as the beginner regression. Progress depth, stance width or duration before optional dumbbell load.</x:v>
+      </x:c>
+      <x:c r="G217" s="5" t="str">
+        <x:v>Take a wide stance and sink straight down between your feet.</x:v>
+      </x:c>
+      <x:c r="H217" s="5" t="str">
+        <x:v>Push knees over toes and keep your torso tall.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Canonicalise Seated Good Morning variants
Agent: yearrepair
</commit_message>
<xml_diff>
--- a/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
+++ b/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="R1fe7015252624050"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Rf85d991d96a94cd3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -433,7 +433,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>CHANGE LOG — Sam 2026-07-27: MetCon row DELETED (the conditioning ruling retiring the name wins); Single-Arm Pulldown row ADDED (Lats / Upper back, Midline / everyone); 3 casing typos corrected as authorised edits (Suitcase Carry + Skull Crushers 'Everyone' -&gt; 'everyone', Chin-Up Negative (Slow) secondary 'midline' -&gt; 'Midline'). CHANGE LOG — 2026-07-28 cue reconciliation: renamed from MUSCLE_EXPERIENCE_FINAL_2026-07-25.xlsx; primaryCue/secondaryCue columns added, making this the single authored source for coaching cues. 175 rows carry Sam-authored cues as shipped; 23 conditioning rows read "PENDING — Stage B" (unruled, NOT blessed — Sam 2026-07-28). Muscle/experience cells are untouched. CHANGE LOG — 2026-09-01 identity merge: Single-Arm Pulldown retired as a current row and retained only as a legacy read alias; cues, equipment, progression and history resolve to Single-Arm Lat Pulldown.</x:v>
+        <x:v>CHANGE LOG — Sam 2026-07-27: MetCon row DELETED (the conditioning ruling retiring the name wins); Single-Arm Pulldown row ADDED (Lats / Upper back, Midline / everyone); 3 casing typos corrected as authorised edits (Suitcase Carry + Skull Crushers 'Everyone' -&gt; 'everyone', Chin-Up Negative (Slow) secondary 'midline' -&gt; 'Midline'). CHANGE LOG — 2026-07-28 cue reconciliation: renamed from MUSCLE_EXPERIENCE_FINAL_2026-07-25.xlsx; primaryCue/secondaryCue columns added, making this the single authored source for coaching cues. 175 rows carry Sam-authored cues as shipped; 23 conditioning rows read "PENDING — Stage B" (unruled, NOT blessed — Sam 2026-07-28). Muscle/experience cells are untouched. CHANGE LOG — 2026-09-01 identity merge: Single-Arm Pulldown retired as a current row and retained only as a legacy read alias; cues, equipment, progression and history resolve to Single-Arm Lat Pulldown. CHANGE LOG — 2026-09-01: Seated Good Morning (Barbell) retired as a current row and retained only as legacy saved-data ingress. Seated Good Morning is the one identity; bodyweight is available to everyone, while dumbbell and barbell variants require 1+ years.</x:v>
       </x:c>
       <x:c r="B5"/>
       <x:c r="C5"/>
@@ -5328,7 +5328,7 @@
         <x:v>everyone</x:v>
       </x:c>
       <x:c r="F208" s="5" t="str">
-        <x:v>Lower for 5 seconds. Bodyweight mobility; never a main lift.</x:v>
+        <x:v>Lower for 5 seconds. Bodyweight for everyone; dumbbell and barbell variants require 1+ years. Log total external load. Mobility only; never a main lift.</x:v>
       </x:c>
       <x:c r="G208" s="5" t="str">
         <x:v>Sit wide, brace, and hinge forward from the hips.</x:v>
@@ -5496,52 +5496,36 @@
         <x:v>Mobility</x:v>
       </x:c>
       <x:c r="B215" s="5" t="str">
-        <x:v>Seated Good Morning (Barbell)</x:v>
+        <x:v>Horse Stance Hold</x:v>
       </x:c>
       <x:c r="C215" s="5" t="str">
-        <x:v>Low back, Groin</x:v>
+        <x:v>Groin, Quads, Glutes</x:v>
       </x:c>
       <x:c r="D215" s="5" t="str">
-        <x:v>Hamstrings, Glutes, Midline, Upper back</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E215" s="5" t="str">
-        <x:v>1+ years</x:v>
+        <x:v>everyone</x:v>
       </x:c>
       <x:c r="F215" s="5" t="str">
-        <x:v>Lower for 5 seconds. Start with an empty bar; log total external load. Mobility only; excluded the day before a game.</x:v>
+        <x:v>2 × 60-second total holds. Bodyweight; use a higher or narrower stance as the beginner regression. Progress depth, stance width or duration before optional dumbbell load.</x:v>
       </x:c>
       <x:c r="G215" s="5" t="str">
-        <x:v>Sit wide, brace, and hinge forward from the hips.</x:v>
+        <x:v>Take a wide stance and sink straight down between your feet.</x:v>
       </x:c>
       <x:c r="H215" s="5" t="str">
-        <x:v>Don't round the spine.</x:v>
+        <x:v>Push knees over toes and keep your torso tall.</x:v>
       </x:c>
     </x:row>
     <x:row r="216" ht="70" customHeight="1">
-      <x:c r="A216" s="5" t="str">
-        <x:v>Mobility</x:v>
-      </x:c>
-      <x:c r="B216" s="5" t="str">
-        <x:v>Horse Stance Hold</x:v>
-      </x:c>
-      <x:c r="C216" s="5" t="str">
-        <x:v>Groin, Quads, Glutes</x:v>
-      </x:c>
-      <x:c r="D216" s="5" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E216" s="5" t="str">
-        <x:v>everyone</x:v>
-      </x:c>
-      <x:c r="F216" s="5" t="str">
-        <x:v>2 × 60-second total holds. Bodyweight; use a higher or narrower stance as the beginner regression. Progress depth, stance width or duration before optional dumbbell load.</x:v>
-      </x:c>
-      <x:c r="G216" s="5" t="str">
-        <x:v>Take a wide stance and sink straight down between your feet.</x:v>
-      </x:c>
-      <x:c r="H216" s="5" t="str">
-        <x:v>Push knees over toes and keep your torso tall.</x:v>
-      </x:c>
+      <x:c r="A216" s="5"/>
+      <x:c r="B216" s="5"/>
+      <x:c r="C216" s="5"/>
+      <x:c r="D216" s="5"/>
+      <x:c r="E216" s="5"/>
+      <x:c r="F216" s="5"/>
+      <x:c r="G216" s="5"/>
+      <x:c r="H216" s="5"/>
     </x:row>
     <x:row r="217" ht="90" customHeight="1">
       <x:c r="A217" s="5"/>

</xml_diff>

<commit_message>
Move hamstring work into lower prehab
Agent: lowerprehab
</commit_message>
<xml_diff>
--- a/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
+++ b/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Rf85d991d96a94cd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Rd4cc36d77d894aea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -433,7 +433,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>CHANGE LOG — Sam 2026-07-27: MetCon row DELETED (the conditioning ruling retiring the name wins); Single-Arm Pulldown row ADDED (Lats / Upper back, Midline / everyone); 3 casing typos corrected as authorised edits (Suitcase Carry + Skull Crushers 'Everyone' -&gt; 'everyone', Chin-Up Negative (Slow) secondary 'midline' -&gt; 'Midline'). CHANGE LOG — 2026-07-28 cue reconciliation: renamed from MUSCLE_EXPERIENCE_FINAL_2026-07-25.xlsx; primaryCue/secondaryCue columns added, making this the single authored source for coaching cues. 175 rows carry Sam-authored cues as shipped; 23 conditioning rows read "PENDING — Stage B" (unruled, NOT blessed — Sam 2026-07-28). Muscle/experience cells are untouched. CHANGE LOG — 2026-09-01 identity merge: Single-Arm Pulldown retired as a current row and retained only as a legacy read alias; cues, equipment, progression and history resolve to Single-Arm Lat Pulldown. CHANGE LOG — 2026-09-01: Seated Good Morning (Barbell) retired as a current row and retained only as legacy saved-data ingress. Seated Good Morning is the one identity; bodyweight is available to everyone, while dumbbell and barbell variants require 1+ years.</x:v>
+        <x:v>CHANGE LOG — Sam 2026-07-27: MetCon row DELETED (the conditioning ruling retiring the name wins); Single-Arm Pulldown row ADDED (Lats / Upper back, Midline / everyone); 3 casing typos corrected as authorised edits (Suitcase Carry + Skull Crushers 'Everyone' -&gt; 'everyone', Chin-Up Negative (Slow) secondary 'midline' -&gt; 'Midline'). CHANGE LOG — 2026-07-28 cue reconciliation: renamed from MUSCLE_EXPERIENCE_FINAL_2026-07-25.xlsx; primaryCue/secondaryCue columns added, making this the single authored source for coaching cues. 175 rows carry Sam-authored cues as shipped; 23 conditioning rows read "PENDING — Stage B" (unruled, NOT blessed — Sam 2026-07-28). Muscle/experience cells are untouched. CHANGE LOG — 2026-09-01 identity merge: Single-Arm Pulldown retired as a current row and retained only as a legacy read alias; cues, equipment, progression and history resolve to Single-Arm Lat Pulldown. CHANGE LOG — 2026-09-01: Seated Good Morning (Barbell) retired as a current row and retained only as legacy saved-data ingress. Seated Good Morning is the one identity; bodyweight is available to everyone, while dumbbell and barbell variants require 1+ years.; Sam 2026-09-02: SL 45° Back Extension Hold and Swiss Ball Hamstring Curl moved from Hamstring (light) into Lower prehab; the separate authored pool was retired.</x:v>
       </x:c>
       <x:c r="B5"/>
       <x:c r="C5"/>
@@ -3311,7 +3311,7 @@
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="1" t="str">
-        <x:v>Hamstring (light)</x:v>
+        <x:v>Lower prehab</x:v>
       </x:c>
       <x:c r="B125" s="1" t="str">
         <x:v>Swiss Ball Hamstring Curl</x:v>
@@ -5365,7 +5365,7 @@
     </x:row>
     <x:row r="210" ht="70" customHeight="1">
       <x:c r="A210" s="5" t="str">
-        <x:v>Hamstring (light)</x:v>
+        <x:v>Lower prehab</x:v>
       </x:c>
       <x:c r="B210" s="5" t="str">
         <x:v>SL 45° Back Extension Hold</x:v>

</xml_diff>

<commit_message>
Add Bench Thoracic Extension
Agent: benchthoracic
</commit_message>
<xml_diff>
--- a/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
+++ b/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Rd4cc36d77d894aea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="R4733d448f61a412d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5518,14 +5518,30 @@
       </x:c>
     </x:row>
     <x:row r="216" ht="70" customHeight="1">
-      <x:c r="A216" s="5"/>
-      <x:c r="B216" s="5"/>
-      <x:c r="C216" s="5"/>
-      <x:c r="D216" s="5"/>
-      <x:c r="E216" s="5"/>
-      <x:c r="F216" s="5"/>
-      <x:c r="G216" s="5"/>
-      <x:c r="H216" s="5"/>
+      <x:c r="A216" s="5" t="str">
+        <x:v>Mobility</x:v>
+      </x:c>
+      <x:c r="B216" s="5" t="str">
+        <x:v>Bench Thoracic Extension</x:v>
+      </x:c>
+      <x:c r="C216" s="5" t="str">
+        <x:v>Lats, Upper back</x:v>
+      </x:c>
+      <x:c r="D216" s="5" t="str">
+        <x:v>Triceps, Chest, Midline</x:v>
+      </x:c>
+      <x:c r="E216" s="5" t="str">
+        <x:v>everyone</x:v>
+      </x:c>
+      <x:c r="F216" s="5" t="str">
+        <x:v>Slow reps. Pause 3 seconds at the bottom. Bodyweight only; use a comfortable range near games.</x:v>
+      </x:c>
+      <x:c r="G216" s="5" t="str">
+        <x:v>Place elbows on the bench and sit your hips back.</x:v>
+      </x:c>
+      <x:c r="H216" s="5" t="str">
+        <x:v>Sink your chest without arching through the lower back.</x:v>
+      </x:c>
     </x:row>
     <x:row r="217" ht="90" customHeight="1">
       <x:c r="A217" s="5"/>

</xml_diff>

<commit_message>
Add Sleeper Stretch and RFE Split Squat Jump
Agent: sleeperstretch
</commit_message>
<xml_diff>
--- a/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
+++ b/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="R4733d448f61a412d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Rf8f1d2c807e34470"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5152,7 +5152,7 @@
         <x:v>2+ years</x:v>
       </x:c>
       <x:c r="F201" s="1" t="str">
-        <x:v>FLAG — gate proposed, confirm</x:v>
+        <x:v>Auto lower power. Bench; 2+ years. Not in-season or near games.</x:v>
       </x:c>
       <x:c r="G201" s="1" t="str">
         <x:v>Back foot on bench, slight lean forward, jump straight up off the front leg.</x:v>
@@ -5544,14 +5544,30 @@
       </x:c>
     </x:row>
     <x:row r="217" ht="90" customHeight="1">
-      <x:c r="A217" s="5"/>
-      <x:c r="B217" s="5"/>
-      <x:c r="C217" s="5"/>
-      <x:c r="D217" s="5"/>
-      <x:c r="E217" s="5"/>
-      <x:c r="F217" s="5"/>
-      <x:c r="G217" s="5"/>
-      <x:c r="H217" s="5"/>
+      <x:c r="A217" s="5" t="str">
+        <x:v>Mobility</x:v>
+      </x:c>
+      <x:c r="B217" s="5" t="str">
+        <x:v>Sleeper Stretch</x:v>
+      </x:c>
+      <x:c r="C217" s="5" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="D217" s="5" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E217" s="5" t="str">
+        <x:v>everyone</x:v>
+      </x:c>
+      <x:c r="F217" s="5" t="str">
+        <x:v>Gentle pressure from the opposite hand; no external loading or bouncing. Use short, comfortable holds near games and avoid aggressive holds before throwing, pressing or contact.</x:v>
+      </x:c>
+      <x:c r="G217" s="5" t="str">
+        <x:v>Lie on the target shoulder and gently lower the forearm.</x:v>
+      </x:c>
+      <x:c r="H217" s="5" t="str">
+        <x:v>Stop at a mild stretch behind the shoulder, never the front.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add Foam Roller Thoracic Extension
Agent: foamthoracic
</commit_message>
<xml_diff>
--- a/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
+++ b/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Rf8f1d2c807e34470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Rd47f9b569f604df7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5569,6 +5569,32 @@
         <x:v>Stop at a mild stretch behind the shoulder, never the front.</x:v>
       </x:c>
     </x:row>
+    <x:row r="218">
+      <x:c r="A218" s="5" t="str">
+        <x:v>Mobility</x:v>
+      </x:c>
+      <x:c r="B218" s="5" t="str">
+        <x:v>Foam Roller Thoracic Extension</x:v>
+      </x:c>
+      <x:c r="C218" s="5" t="str">
+        <x:v>Lats, Upper back</x:v>
+      </x:c>
+      <x:c r="D218" s="5" t="str">
+        <x:v>Chest, Triceps, Shoulders, Midline</x:v>
+      </x:c>
+      <x:c r="E218" s="5" t="str">
+        <x:v>everyone</x:v>
+      </x:c>
+      <x:c r="F218" s="5" t="str">
+        <x:v>Pause 5 seconds overhead. Foam roller required. Hold one light dumbbell or weight plate in both hands; record total load. Beginners may use no weight. Mobility only; the weight assists the stretch.</x:v>
+      </x:c>
+      <x:c r="G218" s="5" t="str">
+        <x:v>Reach the weight overhead as your upper back extends.</x:v>
+      </x:c>
+      <x:c r="H218" s="5" t="str">
+        <x:v>Keep ribs tucked and avoid arching through the lower back.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add Incline Push-Up and Single-Leg Hop and Stick
Working: source-bound Push-ups regression and 2+ years lower-power option, with master-sheet, cues, equipment, load, injury and dose records. Focused intake 913/913 including eight mutations; power 104/104; muscle/workbook 97/97 over 214 rows; equipment 95/95; automatic weekly selection 13/13; quick actions 64/64. Product/dev compile 0; seven unrelated test-only errors remain. Law registry 238 guarded of 259, with 21 older UNENFORCED rows. NOT COVERED: clinical validation, external video playback, and physical-iPhone acceptance. Agent: inclinehop
</commit_message>
<xml_diff>
--- a/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
+++ b/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="R2165b7fe4e7e4596"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="R96c1c2d09ec24480"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5621,6 +5621,58 @@
         <x:v>Lower under control until your elbows fully straighten.</x:v>
       </x:c>
     </x:row>
+    <x:row r="220" ht="72" customHeight="1">
+      <x:c r="A220" s="5" t="str">
+        <x:v>Upper push horizontal</x:v>
+      </x:c>
+      <x:c r="B220" s="5" t="str">
+        <x:v>Incline Push-Up</x:v>
+      </x:c>
+      <x:c r="C220" s="5" t="str">
+        <x:v>Chest, Triceps, Shoulders</x:v>
+      </x:c>
+      <x:c r="D220" s="5" t="str">
+        <x:v>Midline, Glutes</x:v>
+      </x:c>
+      <x:c r="E220" s="5" t="str">
+        <x:v>everyone (regression)</x:v>
+      </x:c>
+      <x:c r="F220" s="5" t="str">
+        <x:v>Automatic regression and manual Swap from Push-ups only. Eligible for all complete beginners and female athletes at 1–2 years. Requires a bench or plyo box. Bodyweight only; record support height in the session note and lower it to progress. Inherits Push-ups sets, reps and role. All phases; suitable near games.</x:v>
+      </x:c>
+      <x:c r="G220" s="5" t="str">
+        <x:v>Keep a straight body line and lower your chest to the support.</x:v>
+      </x:c>
+      <x:c r="H220" s="5" t="str">
+        <x:v>Press away without letting your hips sag or shoulders shrug.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="72" customHeight="1">
+      <x:c r="A221" s="5" t="str">
+        <x:v>Power</x:v>
+      </x:c>
+      <x:c r="B221" s="5" t="str">
+        <x:v>Single-Leg Hop and Stick</x:v>
+      </x:c>
+      <x:c r="C221" s="5" t="str">
+        <x:v>Glutes, Quads, Calves</x:v>
+      </x:c>
+      <x:c r="D221" s="5" t="str">
+        <x:v>Hamstrings, Groin, Midline, Feet</x:v>
+      </x:c>
+      <x:c r="E221" s="5" t="str">
+        <x:v>2+ years</x:v>
+      </x:c>
+      <x:c r="F221" s="5" t="str">
+        <x:v>Automatic lower power and manual Add/Swap for 2+ years only. Bodyweight; 2 × 5 per side with 120 seconds rest. All phases and in-season at low volume; never automatic at G-1. Progress hop distance only while the landing stays controlled.</x:v>
+      </x:c>
+      <x:c r="G221" s="5" t="str">
+        <x:v>Hop forward from one leg and freeze the landing.</x:v>
+      </x:c>
+      <x:c r="H221" s="5" t="str">
+        <x:v>Land quietly, absorb through the hip, and hold your balance.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(programming): add typed movement-plane metadata
Agent: movementplane
</commit_message>
<xml_diff>
--- a/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
+++ b/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="R96c1c2d09ec24480"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Raa44463d67934fa0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -381,9 +381,11 @@
     <x:col min="6" max="6" width="50" customWidth="1"/>
     <x:col min="7" max="7" width="60" customWidth="1"/>
     <x:col min="8" max="8" width="60" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="4" t="str">
         <x:v>AUTHORED FINAL — Sam sign-off 2026-07-25. Source of truth for the D11 muscle-block build. Changes require Sam.</x:v>
       </x:c>
@@ -394,8 +396,14 @@
       <x:c r="F1"/>
       <x:c r="G1"/>
       <x:c r="H1"/>
-    </x:row>
-    <x:row r="2">
+      <x:c r="I1" s="5" t="str">
+        <x:v>MOVEMENT PLANES — 2026-09-02</x:v>
+      </x:c>
+      <x:c r="J1" s="5" t="str">
+        <x:v>Blank = unanswered</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="1" t="str">
         <x:v>EXPERIENCE VALUES: everyone · everyone (regression) · 1+ years · 2+ years · advanced only</x:v>
       </x:c>
@@ -406,6 +414,12 @@
       <x:c r="F2" s="1"/>
       <x:c r="G2"/>
       <x:c r="H2"/>
+      <x:c r="I2" s="5" t="str">
+        <x:v>sagittal · frontal · transverse</x:v>
+      </x:c>
+      <x:c r="J2" s="5" t="str">
+        <x:v>multiplanar · not_applicable</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
@@ -418,6 +432,8 @@
       <x:c r="F3" s="1"/>
       <x:c r="G3"/>
       <x:c r="H3"/>
+      <x:c r="I3"/>
+      <x:c r="J3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="1" t="str">
@@ -430,6 +446,8 @@
       <x:c r="F4" s="1"/>
       <x:c r="G4"/>
       <x:c r="H4"/>
+      <x:c r="I4"/>
+      <x:c r="J4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
@@ -442,6 +460,8 @@
       <x:c r="F5"/>
       <x:c r="G5"/>
       <x:c r="H5"/>
+      <x:c r="I5"/>
+      <x:c r="J5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="2" t="str">
@@ -468,6 +488,12 @@
       <x:c r="H6" s="2" t="str">
         <x:v>secondaryCue</x:v>
       </x:c>
+      <x:c r="I6" s="5" t="str">
+        <x:v>Primary Plane</x:v>
+      </x:c>
+      <x:c r="J6" s="5" t="str">
+        <x:v>Secondary Plane(s)</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1" t="str">
@@ -492,6 +518,10 @@
       <x:c r="H7" s="1" t="str">
         <x:v>Own the bottom position.</x:v>
       </x:c>
+      <x:c r="I7" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J7" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="str">
@@ -518,6 +548,10 @@
       <x:c r="H8" s="1" t="str">
         <x:v>Stay tall through the midline.</x:v>
       </x:c>
+      <x:c r="I8" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J8" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="str">
@@ -542,6 +576,10 @@
       <x:c r="H9" s="1" t="str">
         <x:v>Explode off the box.</x:v>
       </x:c>
+      <x:c r="I9" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J9" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="1" t="str">
@@ -564,6 +602,10 @@
         <x:v>High box to minimise soreness, slight pause at box, stay tight through midline.</x:v>
       </x:c>
       <x:c r="H10" s="1" t="str"/>
+      <x:c r="I10" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J10" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="str">
@@ -588,6 +630,12 @@
       <x:c r="H11" s="1" t="str">
         <x:v>Steady and deliberate.</x:v>
       </x:c>
+      <x:c r="I11" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1" t="str">
@@ -612,6 +660,12 @@
       <x:c r="H12" s="1" t="str">
         <x:v>Control the descent, no bouncing.</x:v>
       </x:c>
+      <x:c r="I12" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1" t="str">
@@ -636,6 +690,12 @@
       <x:c r="H13" s="1" t="str">
         <x:v>Front knee tracks over the toe.</x:v>
       </x:c>
+      <x:c r="I13" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1" t="str">
@@ -660,6 +720,12 @@
       <x:c r="H14" s="1" t="str">
         <x:v>Don’t bounce with leg on ground.</x:v>
       </x:c>
+      <x:c r="I14" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1" t="str">
@@ -684,6 +750,10 @@
       <x:c r="H15" s="1" t="str">
         <x:v>Smooth tempo, no rushing.</x:v>
       </x:c>
+      <x:c r="I15" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J15" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1" t="str">
@@ -708,6 +778,10 @@
       <x:c r="H16" s="1" t="str">
         <x:v>Push through the whole foot.</x:v>
       </x:c>
+      <x:c r="I16" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J16" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="1" t="str">
@@ -732,6 +806,10 @@
       <x:c r="H17" s="1" t="str">
         <x:v>Control on the way down.</x:v>
       </x:c>
+      <x:c r="I17" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J17" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="1" t="str">
@@ -756,6 +834,12 @@
       <x:c r="H18" s="1" t="str">
         <x:v>Keep the knee tracking straight.</x:v>
       </x:c>
+      <x:c r="I18" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>frontal, transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="1" t="str">
@@ -776,6 +860,10 @@
         <x:v>Sit back into hips, knees follow toes, chest tall.</x:v>
       </x:c>
       <x:c r="H19" s="1" t="str"/>
+      <x:c r="I19" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J19" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="1" t="str">
@@ -802,6 +890,10 @@
       <x:c r="H20" s="1" t="str">
         <x:v>Flat back from start to lockout.</x:v>
       </x:c>
+      <x:c r="I20" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J20" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="1" t="str">
@@ -826,6 +918,10 @@
       <x:c r="H21" s="1" t="str">
         <x:v>Hips and shoulders rise together.</x:v>
       </x:c>
+      <x:c r="I21" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J21" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="1" t="str">
@@ -852,6 +948,10 @@
       <x:c r="H22" s="1" t="str">
         <x:v>Feel the hamstrings load on the way down.</x:v>
       </x:c>
+      <x:c r="I22" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J22" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="1" t="str">
@@ -876,6 +976,12 @@
       <x:c r="H23" s="1" t="str">
         <x:v>Balance and control over speed.</x:v>
       </x:c>
+      <x:c r="I23" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J23" t="str">
+        <x:v>frontal, transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="1" t="str">
@@ -900,6 +1006,10 @@
       <x:c r="H24" s="1" t="str">
         <x:v>Ribs down, no overextending.</x:v>
       </x:c>
+      <x:c r="I24" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J24" t="str"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="1" t="str">
@@ -924,6 +1034,10 @@
       <x:c r="H25" s="1" t="str">
         <x:v>Power from hips, don’t lift with arms.</x:v>
       </x:c>
+      <x:c r="I25" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J25" t="str"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="1" t="str">
@@ -946,6 +1060,10 @@
         <x:v>Keep spine neutral, don’t arch low back, lift hips, squeeze glutes, add weight to hips if you can.</x:v>
       </x:c>
       <x:c r="H26" s="1" t="str"/>
+      <x:c r="I26" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J26" t="str"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="1" t="str">
@@ -970,6 +1088,10 @@
       <x:c r="H27" s="1" t="str">
         <x:v>Bar to chest, press hard to lockout.</x:v>
       </x:c>
+      <x:c r="I27" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J27" t="str"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="1" t="str">
@@ -994,6 +1116,12 @@
       <x:c r="H28" s="1" t="str">
         <x:v>Press through the palms.</x:v>
       </x:c>
+      <x:c r="I28" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J28" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="1" t="str">
@@ -1018,6 +1146,12 @@
       <x:c r="H29" s="1" t="str">
         <x:v>Triceps do the work.</x:v>
       </x:c>
+      <x:c r="I29" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J29" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="1" t="str">
@@ -1042,6 +1176,10 @@
       <x:c r="H30" s="1" t="str">
         <x:v>Control the dumbbells down and drive.</x:v>
       </x:c>
+      <x:c r="I30" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J30" t="str"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="1" t="str">
@@ -1066,6 +1204,12 @@
       <x:c r="H31" s="1" t="str">
         <x:v>Drive up and together.</x:v>
       </x:c>
+      <x:c r="I31" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J31" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="1" t="str">
@@ -1090,6 +1234,12 @@
       <x:c r="H32" s="1" t="str">
         <x:v>Chest to floor, full lockout.</x:v>
       </x:c>
+      <x:c r="I32" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J32" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="1" t="str">
@@ -1114,6 +1264,10 @@
       <x:c r="H33" s="1" t="str">
         <x:v>Control the descent.</x:v>
       </x:c>
+      <x:c r="I33" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J33" t="str"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="1" t="str">
@@ -1140,6 +1294,10 @@
       <x:c r="H34" s="1" t="str">
         <x:v>Brace hard through the midline.</x:v>
       </x:c>
+      <x:c r="I34" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J34" t="str"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="1" t="str">
@@ -1166,6 +1324,10 @@
       <x:c r="H35" s="1" t="str">
         <x:v>Don't let the torso rotate.</x:v>
       </x:c>
+      <x:c r="I35" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J35" t="str"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="1" t="str">
@@ -1190,6 +1352,12 @@
       <x:c r="H36" s="1" t="str">
         <x:v>Press hard and finish strong.</x:v>
       </x:c>
+      <x:c r="I36" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J36" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="1" t="str">
@@ -1216,6 +1384,12 @@
       <x:c r="H37" s="1" t="str">
         <x:v>Stable base, strong finish.</x:v>
       </x:c>
+      <x:c r="I37" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J37" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="1" t="str">
@@ -1240,6 +1414,12 @@
       <x:c r="H38" s="1" t="str">
         <x:v>No arching through the lower back.</x:v>
       </x:c>
+      <x:c r="I38" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J38" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="1" t="str">
@@ -1264,6 +1444,12 @@
       <x:c r="H39" s="1" t="str">
         <x:v>Ribs down, control the descent.</x:v>
       </x:c>
+      <x:c r="I39" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J39" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="1" t="str">
@@ -1288,6 +1474,12 @@
       <x:c r="H40" s="1" t="str">
         <x:v>Fight the rotation, ribs stay down.</x:v>
       </x:c>
+      <x:c r="I40" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J40" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="1" t="str">
@@ -1312,6 +1504,8 @@
       <x:c r="H41" s="1" t="str">
         <x:v>Full lockout, reset quickly.</x:v>
       </x:c>
+      <x:c r="I41"/>
+      <x:c r="J41"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="1" t="str">
@@ -1338,6 +1532,12 @@
       <x:c r="H42" s="1" t="str">
         <x:v>Stay tight through midline. Can be done seated on a bench, or with dumbbells.</x:v>
       </x:c>
+      <x:c r="I42" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J42" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="1" t="str">
@@ -1362,6 +1562,12 @@
       <x:c r="H43" s="1" t="str">
         <x:v>Squeeze the shoulder blades at the top.</x:v>
       </x:c>
+      <x:c r="I43" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J43" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="1" t="str">
@@ -1388,6 +1594,12 @@
       <x:c r="H44" s="1" t="str">
         <x:v>Retract and hold for a beat.</x:v>
       </x:c>
+      <x:c r="I44" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J44" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="1" t="str">
@@ -1412,6 +1624,12 @@
       <x:c r="H45" s="1" t="str">
         <x:v>Keep the hips and shoulders square.</x:v>
       </x:c>
+      <x:c r="I45" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J45" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="1" t="str">
@@ -1436,6 +1654,12 @@
       <x:c r="H46" s="1" t="str">
         <x:v>Slow on the return.</x:v>
       </x:c>
+      <x:c r="I46" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J46" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="1" t="str">
@@ -1460,6 +1684,12 @@
       <x:c r="H47" s="1" t="str">
         <x:v>Squeeze the rear delts, slow return.</x:v>
       </x:c>
+      <x:c r="I47" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J47" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="1" t="str">
@@ -1484,6 +1714,10 @@
       <x:c r="H48" s="1" t="str">
         <x:v>Light weight, feel the squeeze.</x:v>
       </x:c>
+      <x:c r="I48" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J48" t="str"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="1" t="str">
@@ -1508,6 +1742,10 @@
       <x:c r="H49" s="1" t="str">
         <x:v>Elbows straight, controlled return.</x:v>
       </x:c>
+      <x:c r="I49" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J49" t="str"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="1" t="str">
@@ -1532,6 +1770,12 @@
       <x:c r="H50" s="1" t="str">
         <x:v>Initiate with the lats, not the arms. Add weight once bodyweight sets feel easy.</x:v>
       </x:c>
+      <x:c r="I50" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J50" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="1" t="str">
@@ -1556,6 +1800,12 @@
       <x:c r="H51" s="1" t="str">
         <x:v>Control the lowering.</x:v>
       </x:c>
+      <x:c r="I51" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J51" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="1" t="str">
@@ -1580,6 +1830,12 @@
       <x:c r="H52" s="1" t="str">
         <x:v>Squeeze at the bottom, slow return.</x:v>
       </x:c>
+      <x:c r="I52" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J52" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="1" t="str">
@@ -1602,6 +1858,12 @@
         <x:v>Use V grip attachment, puff chest out as hands come down.</x:v>
       </x:c>
       <x:c r="H53" s="1" t="str"/>
+      <x:c r="I53" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J53" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="1" t="str">
@@ -1628,6 +1890,12 @@
       <x:c r="H54" s="1" t="str">
         <x:v>Stay tight through the midline; control the return to a full stretch.</x:v>
       </x:c>
+      <x:c r="I54" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J54" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="1" t="str">
@@ -1652,6 +1920,10 @@
       <x:c r="H55" s="1" t="str">
         <x:v>Land soft, absorb with the hips.</x:v>
       </x:c>
+      <x:c r="I55" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J55" t="str"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="1" t="str">
@@ -1676,6 +1948,10 @@
       <x:c r="H56" s="1" t="str">
         <x:v>Stick the landing.</x:v>
       </x:c>
+      <x:c r="I56" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J56" t="str"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="1" t="str">
@@ -1700,6 +1976,10 @@
       <x:c r="H57" s="1" t="str">
         <x:v>Land soft, reset between reps.</x:v>
       </x:c>
+      <x:c r="I57" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J57" t="str"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="1" t="str">
@@ -1726,6 +2006,12 @@
       <x:c r="H58" s="1" t="str">
         <x:v>Stick each landing before the next.</x:v>
       </x:c>
+      <x:c r="I58" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J58" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="1" t="str">
@@ -1752,6 +2038,12 @@
       <x:c r="H59" s="1" t="str">
         <x:v>Minimum ground contact time.</x:v>
       </x:c>
+      <x:c r="I59" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J59" t="str">
+        <x:v>frontal, transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="1" t="str">
@@ -1776,6 +2068,12 @@
       <x:c r="H60" s="1" t="str">
         <x:v>Breathe and keep moving. Weight shown is per hand.</x:v>
       </x:c>
+      <x:c r="I60" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J60" t="str">
+        <x:v>frontal, transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="1" t="str">
@@ -1800,6 +2098,12 @@
       <x:c r="H61" s="1" t="str">
         <x:v>Short steady steps, no leaning back.</x:v>
       </x:c>
+      <x:c r="I61" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J61" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="1" t="str">
@@ -1824,6 +2128,12 @@
       <x:c r="H62" s="1" t="str">
         <x:v>Don’t rest weight on thigh.</x:v>
       </x:c>
+      <x:c r="I62" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J62" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="1" t="str">
@@ -1848,6 +2158,12 @@
       <x:c r="H63" s="1" t="str">
         <x:v>Weight shown is per hand.</x:v>
       </x:c>
+      <x:c r="I63" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J63" t="str">
+        <x:v>frontal, transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="1" t="str">
@@ -1872,6 +2188,10 @@
       <x:c r="H64" s="1" t="str">
         <x:v>Squeeze at the top, controlled lower.</x:v>
       </x:c>
+      <x:c r="I64" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J64" t="str"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="1" t="str">
@@ -1898,6 +2218,10 @@
       <x:c r="H65" s="1" t="str">
         <x:v>Full range, elbows stay in place.</x:v>
       </x:c>
+      <x:c r="I65" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J65" t="str"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="1" t="str">
@@ -1922,6 +2246,10 @@
       <x:c r="H66" s="1" t="str">
         <x:v>No swinging, control the bar path.</x:v>
       </x:c>
+      <x:c r="I66" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J66" t="str"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="1" t="str">
@@ -1946,6 +2274,10 @@
       <x:c r="H67" s="1" t="str">
         <x:v>Smooth tempo, squeeze at the top.</x:v>
       </x:c>
+      <x:c r="I67" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J67" t="str"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="1" t="str">
@@ -1970,6 +2302,10 @@
       <x:c r="H68" s="1" t="str">
         <x:v>Control both directions.</x:v>
       </x:c>
+      <x:c r="I68" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J68" t="str"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="1" t="str">
@@ -1994,6 +2330,10 @@
       <x:c r="H69" s="1" t="str">
         <x:v>Slow curl, squeeze at the top.</x:v>
       </x:c>
+      <x:c r="I69" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J69" t="str"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="1" t="str">
@@ -2018,6 +2358,10 @@
       <x:c r="H70" s="1" t="str">
         <x:v>Control both directions, no momentum.</x:v>
       </x:c>
+      <x:c r="I70" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J70" t="str"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="1" t="str">
@@ -2044,6 +2388,10 @@
       <x:c r="H71" s="1" t="str">
         <x:v>Slow on the way down.</x:v>
       </x:c>
+      <x:c r="I71" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J71" t="str"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="1" t="str">
@@ -2068,6 +2416,10 @@
       <x:c r="H72" s="1" t="str">
         <x:v>Strict curl, no body swing.</x:v>
       </x:c>
+      <x:c r="I72" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J72" t="str"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="1" t="str">
@@ -2092,6 +2444,10 @@
       <x:c r="H73" s="1" t="str">
         <x:v>Constant tension, no jerking.</x:v>
       </x:c>
+      <x:c r="I73" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J73" t="str"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="1" t="str">
@@ -2116,6 +2472,10 @@
       <x:c r="H74" s="1" t="str">
         <x:v>Constant tension, no slack.</x:v>
       </x:c>
+      <x:c r="I74" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J74" t="str"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="1" t="str">
@@ -2140,6 +2500,10 @@
       <x:c r="H75" s="1" t="str">
         <x:v>Elbows stay pointed forward.</x:v>
       </x:c>
+      <x:c r="I75" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J75" t="str"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="1" t="str">
@@ -2166,6 +2530,10 @@
       <x:c r="H76" s="1" t="str">
         <x:v>Elbows stay fixed in place.</x:v>
       </x:c>
+      <x:c r="I76" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J76" t="str"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="1" t="str">
@@ -2190,6 +2558,10 @@
       <x:c r="H77" s="1" t="str">
         <x:v>Squeeze at the top, slow return.</x:v>
       </x:c>
+      <x:c r="I77" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J77" t="str"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="1" t="str">
@@ -2214,6 +2586,10 @@
       <x:c r="H78" s="1" t="str">
         <x:v>Empty the triceps by the final rep.</x:v>
       </x:c>
+      <x:c r="I78" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J78" t="str"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="1" t="str">
@@ -2238,6 +2614,10 @@
       <x:c r="H79" s="1" t="str">
         <x:v>No momentum, strict form.</x:v>
       </x:c>
+      <x:c r="I79" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J79" t="str"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="1" t="str">
@@ -2262,6 +2642,12 @@
       <x:c r="H80" s="1" t="str">
         <x:v>Light weight, pause at the top.</x:v>
       </x:c>
+      <x:c r="I80" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J80" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="1" t="str">
@@ -2286,6 +2672,10 @@
       <x:c r="H81" s="1" t="str">
         <x:v>Pause at the top, controlled lower.</x:v>
       </x:c>
+      <x:c r="I81" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J81" t="str"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="1" t="str">
@@ -2312,6 +2702,10 @@
       <x:c r="H82" s="1" t="str">
         <x:v>Fight gravity the whole way down.</x:v>
       </x:c>
+      <x:c r="I82" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J82" t="str"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="1" t="str">
@@ -2334,6 +2728,10 @@
         <x:v>Pad should be lower calf area, squeeze heels to butt.</x:v>
       </x:c>
       <x:c r="H83" s="1" t="str"/>
+      <x:c r="I83" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J83" t="str"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="1" t="str">
@@ -2356,6 +2754,10 @@
         <x:v>Drive feet to ceiling, lean back slightly if possible.</x:v>
       </x:c>
       <x:c r="H84" s="1" t="str"/>
+      <x:c r="I84" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J84" t="str"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="1" t="str">
@@ -2380,6 +2782,10 @@
       <x:c r="H85" s="1" t="str">
         <x:v>Pause high, lower slowly.</x:v>
       </x:c>
+      <x:c r="I85" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J85" t="str"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="1" t="str">
@@ -2406,6 +2812,10 @@
       <x:c r="H86" s="1" t="str">
         <x:v>Controlled reps, full range.</x:v>
       </x:c>
+      <x:c r="I86" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J86" t="str"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="1" t="str">
@@ -2428,6 +2838,12 @@
         <x:v>Upper back on bench, add weight to hips, one leg up, drive hips to sky, squeeze glutes.</x:v>
       </x:c>
       <x:c r="H87" s="1" t="str"/>
+      <x:c r="I87" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J87" t="str">
+        <x:v>frontal, transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="1" t="str">
@@ -2452,6 +2868,10 @@
         <x:v>Squeeze glutes at top, round slightly at bottom.</x:v>
       </x:c>
       <x:c r="H88" s="1" t="str"/>
+      <x:c r="I88" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J88" t="str"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="1" t="str">
@@ -2478,6 +2898,12 @@
       <x:c r="H89" s="1" t="str">
         <x:v>Fight gravity the whole way.</x:v>
       </x:c>
+      <x:c r="I89" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J89" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" t="str">
@@ -2502,6 +2928,12 @@
       <x:c r="H90" s="1" t="str">
         <x:v>Squeeze the rear delts.</x:v>
       </x:c>
+      <x:c r="I90" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J90" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="1" t="str">
@@ -2526,6 +2958,12 @@
       <x:c r="H91" s="1" t="str">
         <x:v>Squeeze the shoulder blades back.</x:v>
       </x:c>
+      <x:c r="I91" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J91" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="1" t="str">
@@ -2550,6 +2988,12 @@
       <x:c r="H92" s="1" t="str">
         <x:v>Scale with foot position.</x:v>
       </x:c>
+      <x:c r="I92" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J92" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="1" t="str">
@@ -2574,6 +3018,12 @@
       <x:c r="H93" s="1" t="str">
         <x:v>Hold tension, no dropping.</x:v>
       </x:c>
+      <x:c r="I93" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J93" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="1" t="str">
@@ -2598,6 +3048,12 @@
       <x:c r="H94" s="1" t="str">
         <x:v>Don’t let hips drop.</x:v>
       </x:c>
+      <x:c r="I94" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J94" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="1" t="str">
@@ -2622,6 +3078,10 @@
       <x:c r="H95" s="1" t="str">
         <x:v>Hold each squeeze for a beat.</x:v>
       </x:c>
+      <x:c r="I95" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J95" t="str"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="1" t="str">
@@ -2646,6 +3106,12 @@
       <x:c r="H96" s="1" t="str">
         <x:v>Heel down, chest up, push back through. Hold rack if needed.</x:v>
       </x:c>
+      <x:c r="I96" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J96" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="1" t="str">
@@ -2670,6 +3136,12 @@
       <x:c r="H97" s="1" t="str">
         <x:v>Knee tracks over toes, drive back to standing.</x:v>
       </x:c>
+      <x:c r="I97" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="1" t="str">
@@ -2694,6 +3166,12 @@
       <x:c r="H98" s="1" t="str">
         <x:v>Three-second lowering.</x:v>
       </x:c>
+      <x:c r="I98" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J98" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="1" t="str">
@@ -2718,6 +3196,10 @@
       <x:c r="H99" s="1" t="str">
         <x:v>Slow tempo, no bouncing.</x:v>
       </x:c>
+      <x:c r="I99" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J99" t="str"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="1" t="str">
@@ -2740,6 +3222,10 @@
         <x:v>Band behind knee, step back for tension, straighten knee and squeeze quads.</x:v>
       </x:c>
       <x:c r="H100" s="1" t="str"/>
+      <x:c r="I100" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J100" t="str"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="1" t="str">
@@ -2762,6 +3248,12 @@
         <x:v>Single or double leg, slight knee bend, drive heel into ground, keep hips high.</x:v>
       </x:c>
       <x:c r="H101" s="1" t="str"/>
+      <x:c r="I101" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J101" t="str">
+        <x:v>frontal, transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="1" t="str">
@@ -2784,6 +3276,10 @@
         <x:v>Band behind knees, tension on bands, sit back into a squat and hold.</x:v>
       </x:c>
       <x:c r="H102" s="1" t="str"/>
+      <x:c r="I102" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J102" t="str"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="1" t="str">
@@ -2806,6 +3302,12 @@
         <x:v>Drive knee forward, tap opposite heel on ground, knee tracks over toes.</x:v>
       </x:c>
       <x:c r="H103" s="1" t="str"/>
+      <x:c r="I103" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J103" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="1" t="str">
@@ -2828,6 +3330,12 @@
         <x:v>Sit back into athletic position, band around feet, push off outside leg, keep knees slightly pointed out.</x:v>
       </x:c>
       <x:c r="H104" s="1" t="str"/>
+      <x:c r="I104" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J104" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="1" t="str">
@@ -2852,6 +3360,10 @@
       <x:c r="H105" s="1" t="str">
         <x:v>Hips stay square, slight knee and hip bend.</x:v>
       </x:c>
+      <x:c r="I105" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J105" t="str"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="1" t="str">
@@ -2878,6 +3390,10 @@
       <x:c r="H106" s="1" t="str">
         <x:v>Opposite arm and leg, slow.</x:v>
       </x:c>
+      <x:c r="I106" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J106" t="str"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="1" t="str">
@@ -2902,6 +3418,10 @@
       <x:c r="H107" s="1" t="str">
         <x:v>Lower back stays glued to the floor.</x:v>
       </x:c>
+      <x:c r="I107" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J107" t="str"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="1" t="str">
@@ -2926,6 +3446,10 @@
       <x:c r="H108" s="1" t="str">
         <x:v>Slow extension, full exhale.</x:v>
       </x:c>
+      <x:c r="I108" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J108" t="str"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="1" t="str">
@@ -2950,6 +3474,10 @@
       <x:c r="H109" s="1" t="str">
         <x:v>Drive low back into hands slightly.</x:v>
       </x:c>
+      <x:c r="I109" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J109" t="str"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="1" t="str">
@@ -2976,6 +3504,10 @@
       <x:c r="H110" s="1" t="str">
         <x:v>Ribs down, slightly rounded back, no sagging at hips.</x:v>
       </x:c>
+      <x:c r="I110" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J110" t="str"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="1" t="str">
@@ -3000,6 +3532,10 @@
       <x:c r="H111" s="1" t="str">
         <x:v>No swinging.</x:v>
       </x:c>
+      <x:c r="I111" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J111" t="str"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="1" t="str">
@@ -3026,6 +3562,12 @@
       <x:c r="H112" s="1" t="str">
         <x:v>Slow and controlled.</x:v>
       </x:c>
+      <x:c r="I112" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J112" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="1" t="str">
@@ -3050,6 +3592,12 @@
       <x:c r="H113" s="1" t="str">
         <x:v>Breathe behind the brace.</x:v>
       </x:c>
+      <x:c r="I113" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J113" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="1" t="str">
@@ -3074,6 +3622,10 @@
         <x:v>Keep spine neutral, brace midline, squeeze butt, breathe.</x:v>
       </x:c>
       <x:c r="H114" s="1" t="str"/>
+      <x:c r="I114" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J114" t="str"/>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="1" t="str">
@@ -3096,6 +3648,10 @@
         <x:v>Stay tight, remember to breathe, low back pinned to floor.</x:v>
       </x:c>
       <x:c r="H115" s="1" t="str"/>
+      <x:c r="I115" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J115" t="str"/>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="1" t="str">
@@ -3118,6 +3674,10 @@
         <x:v>Spine stays neutral, resist rotation through midline.</x:v>
       </x:c>
       <x:c r="H116" s="1" t="str"/>
+      <x:c r="I116" t="str">
+        <x:v>multiplanar</x:v>
+      </x:c>
+      <x:c r="J116" t="str"/>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="1" t="str">
@@ -3142,6 +3702,10 @@
         <x:v>Control the way down, low back should be slightly rounded and roll over ground.</x:v>
       </x:c>
       <x:c r="H117" s="1" t="str"/>
+      <x:c r="I117" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J117" t="str"/>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="1" t="str">
@@ -3164,6 +3728,12 @@
         <x:v>Side plank, row band to top of belly, resist rolling forward.</x:v>
       </x:c>
       <x:c r="H118" s="1" t="str"/>
+      <x:c r="I118" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J118" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="1" t="str">
@@ -3188,6 +3758,12 @@
       <x:c r="H119" s="1" t="str">
         <x:v>Feet stay planted.</x:v>
       </x:c>
+      <x:c r="I119" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J119" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="1" t="str">
@@ -3212,6 +3788,12 @@
       <x:c r="H120" s="1" t="str">
         <x:v>Controlled rotation, not a throw.</x:v>
       </x:c>
+      <x:c r="I120" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J120" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="1" t="str">
@@ -3236,6 +3818,8 @@
       <x:c r="H121" s="1" t="str">
         <x:v>Slow and controlled arc.</x:v>
       </x:c>
+      <x:c r="I121"/>
+      <x:c r="J121"/>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="1" t="str">
@@ -3262,6 +3846,8 @@
       <x:c r="H122" s="1" t="str">
         <x:v>Press smooth, keep ribs down.</x:v>
       </x:c>
+      <x:c r="I122"/>
+      <x:c r="J122"/>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="1" t="str">
@@ -3286,6 +3872,8 @@
       <x:c r="H123" s="1" t="str">
         <x:v>Move slowly, no sagging hips.</x:v>
       </x:c>
+      <x:c r="I123"/>
+      <x:c r="J123"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="1" t="str">
@@ -3308,6 +3896,8 @@
         <x:v>dead hang from bar and relax, pull yourself higher only using your shoulder blades, don't bend arms</x:v>
       </x:c>
       <x:c r="H124" s="1" t="str"/>
+      <x:c r="I124"/>
+      <x:c r="J124"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="1" t="str">
@@ -3332,6 +3922,10 @@
       <x:c r="H125" s="1" t="str">
         <x:v>Curl heels into butt.</x:v>
       </x:c>
+      <x:c r="I125" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J125" t="str"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="1" t="str">
@@ -3356,6 +3950,8 @@
       <x:c r="H126" s="1" t="str">
         <x:v>Relax into the pressure.</x:v>
       </x:c>
+      <x:c r="I126"/>
+      <x:c r="J126"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="1" t="str">
@@ -3380,6 +3976,8 @@
       <x:c r="H127" s="1" t="str">
         <x:v>Open the ribs and breathe.</x:v>
       </x:c>
+      <x:c r="I127"/>
+      <x:c r="J127"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="1" t="str">
@@ -3404,6 +4002,8 @@
       <x:c r="H128" s="1" t="str">
         <x:v>Stack the legs to dial pressure.</x:v>
       </x:c>
+      <x:c r="I128"/>
+      <x:c r="J128"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="1" t="str">
@@ -3428,6 +4028,8 @@
       <x:c r="H129" s="1" t="str">
         <x:v>Roll under the armpit, breathe into it.</x:v>
       </x:c>
+      <x:c r="I129"/>
+      <x:c r="J129"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="1" t="str">
@@ -3452,6 +4054,8 @@
       <x:c r="H130" s="1" t="str">
         <x:v>Breathe through each hold.</x:v>
       </x:c>
+      <x:c r="I130"/>
+      <x:c r="J130"/>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="1" t="str">
@@ -3476,6 +4080,8 @@
       <x:c r="H131" s="1" t="str">
         <x:v>Hold 30-60 seconds per side.</x:v>
       </x:c>
+      <x:c r="I131"/>
+      <x:c r="J131"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="1" t="str">
@@ -3500,6 +4106,8 @@
       <x:c r="H132" s="1" t="str">
         <x:v>Stay tall, shift weight gently.</x:v>
       </x:c>
+      <x:c r="I132"/>
+      <x:c r="J132"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="1" t="str">
@@ -3524,6 +4132,8 @@
       <x:c r="H133" s="1" t="str">
         <x:v>Match each position to a breath.</x:v>
       </x:c>
+      <x:c r="I133"/>
+      <x:c r="J133"/>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="1" t="str">
@@ -3548,6 +4158,8 @@
       <x:c r="H134" s="1" t="str">
         <x:v>Then rotate and reach to the sky.</x:v>
       </x:c>
+      <x:c r="I134"/>
+      <x:c r="J134"/>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="1" t="str">
@@ -3572,6 +4184,8 @@
       <x:c r="H135" s="1" t="str">
         <x:v>Breathe and hold position.</x:v>
       </x:c>
+      <x:c r="I135"/>
+      <x:c r="J135"/>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="1" t="str">
@@ -3596,6 +4210,8 @@
       <x:c r="H136" s="1" t="str">
         <x:v>Tall through the midline, no arching.</x:v>
       </x:c>
+      <x:c r="I136"/>
+      <x:c r="J136"/>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="1" t="str">
@@ -3620,6 +4236,8 @@
       <x:c r="H137" s="1" t="str">
         <x:v>Follow the hand with the eyes.</x:v>
       </x:c>
+      <x:c r="I137"/>
+      <x:c r="J137"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="1" t="str">
@@ -3644,6 +4262,8 @@
       <x:c r="H138" s="1" t="str">
         <x:v>Sink in and breathe.</x:v>
       </x:c>
+      <x:c r="I138"/>
+      <x:c r="J138"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="1" t="str">
@@ -3668,6 +4288,8 @@
       <x:c r="H139" s="1" t="str">
         <x:v>Hold the end range, breathe.</x:v>
       </x:c>
+      <x:c r="I139"/>
+      <x:c r="J139"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="1" t="str">
@@ -3692,6 +4314,8 @@
       <x:c r="H140" s="1" t="str">
         <x:v>Big stretch through the chest, breathe slow.</x:v>
       </x:c>
+      <x:c r="I140"/>
+      <x:c r="J140"/>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="1" t="str">
@@ -3716,6 +4340,8 @@
       <x:c r="H141" s="1" t="str">
         <x:v>Sink the chest, breathe under the armpit, slight lean to one side.</x:v>
       </x:c>
+      <x:c r="I141"/>
+      <x:c r="J141"/>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="1" t="str">
@@ -3740,6 +4366,8 @@
       <x:c r="H142" s="1" t="str">
         <x:v>Breathe - let the spine decompress.</x:v>
       </x:c>
+      <x:c r="I142"/>
+      <x:c r="J142"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="1" t="str">
@@ -3766,6 +4394,8 @@
       <x:c r="H143" s="1" t="str">
         <x:v>Build tolerance gradually.</x:v>
       </x:c>
+      <x:c r="I143"/>
+      <x:c r="J143"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="1" t="str">
@@ -3790,6 +4420,8 @@
       <x:c r="H144" s="1" t="str">
         <x:v>Switch to bent-knee for the soleus.</x:v>
       </x:c>
+      <x:c r="I144"/>
+      <x:c r="J144"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="1" t="str">
@@ -3814,6 +4446,8 @@
         <x:v>Pin legs in 45 deg hyper, bend sideways slowly, don’t push too far, just enough to feel tension.</x:v>
       </x:c>
       <x:c r="H145" s="1" t="str"/>
+      <x:c r="I145"/>
+      <x:c r="J145"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="1" t="str">
@@ -3838,6 +4472,8 @@
         <x:v>Elevate front foot, body stays upright, drive hips to front heel, go slow and pause at bottom.</x:v>
       </x:c>
       <x:c r="H146" s="1" t="str"/>
+      <x:c r="I146"/>
+      <x:c r="J146"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="1" t="str">
@@ -3860,6 +4496,8 @@
         <x:v>Place blocks at level you’re comfortable with, fold forward, bend and straight one leg at a time, slowly.</x:v>
       </x:c>
       <x:c r="H147" s="1" t="str"/>
+      <x:c r="I147"/>
+      <x:c r="J147"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="1" t="str">
@@ -3882,6 +4520,8 @@
         <x:v>Upper back and butt against wall, feet together, knees towards ground, add weight to knee if too easy</x:v>
       </x:c>
       <x:c r="H148" s="1" t="str"/>
+      <x:c r="I148"/>
+      <x:c r="J148"/>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="1" t="str">
@@ -3904,6 +4544,8 @@
         <x:v>Keep back neutral, lift outside leg out and up, can use bent leg to start</x:v>
       </x:c>
       <x:c r="H149" s="1" t="str"/>
+      <x:c r="I149"/>
+      <x:c r="J149"/>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="1" t="str">
@@ -3926,6 +4568,8 @@
         <x:v>Tuck your chin and slowly roll down one segment at a time. Add small weight when easy</x:v>
       </x:c>
       <x:c r="H150" s="1" t="str"/>
+      <x:c r="I150"/>
+      <x:c r="J150"/>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="1" t="str">
@@ -3948,6 +4592,8 @@
         <x:v>Rest upper back on bench, dumbbell over, don't allow ribs to flare up, pause at end range</x:v>
       </x:c>
       <x:c r="H151" s="1" t="str"/>
+      <x:c r="I151"/>
+      <x:c r="J151"/>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="1" t="str">
@@ -3972,6 +4618,8 @@
       <x:c r="H152" s="1" t="str">
         <x:v>This is blood flow, not training.</x:v>
       </x:c>
+      <x:c r="I152"/>
+      <x:c r="J152"/>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="1" t="str">
@@ -3996,6 +4644,8 @@
       <x:c r="H153" s="1" t="str">
         <x:v>No holding the rails.</x:v>
       </x:c>
+      <x:c r="I153"/>
+      <x:c r="J153"/>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="1" t="str">
@@ -4020,6 +4670,8 @@
       <x:c r="H154" s="1" t="str">
         <x:v>Get outside and move.</x:v>
       </x:c>
+      <x:c r="I154"/>
+      <x:c r="J154"/>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="1" t="str">
@@ -4044,6 +4696,8 @@
       <x:c r="H155" s="1" t="str">
         <x:v>Pause at the bottom of each breath.</x:v>
       </x:c>
+      <x:c r="I155"/>
+      <x:c r="J155"/>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="1" t="str">
@@ -4068,6 +4722,8 @@
       <x:c r="H156" s="1" t="str">
         <x:v>Feel the floor push back on the exhale.</x:v>
       </x:c>
+      <x:c r="I156"/>
+      <x:c r="J156"/>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="1" t="str">
@@ -4092,6 +4748,8 @@
       <x:c r="H157" s="1" t="str">
         <x:v>Stay relaxed, find the rhythm.</x:v>
       </x:c>
+      <x:c r="I157"/>
+      <x:c r="J157"/>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="1" t="str">
@@ -4116,6 +4774,8 @@
       <x:c r="H158" s="1" t="str">
         <x:v>Slow breaths into the back.</x:v>
       </x:c>
+      <x:c r="I158"/>
+      <x:c r="J158"/>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="1" t="str">
@@ -4142,6 +4802,8 @@
       <x:c r="H159" s="1" t="str">
         <x:v>Full recovery between efforts.</x:v>
       </x:c>
+      <x:c r="I159"/>
+      <x:c r="J159"/>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="1" t="str">
@@ -4168,6 +4830,8 @@
       <x:c r="H160" s="1" t="str">
         <x:v>Walk back for full recovery.</x:v>
       </x:c>
+      <x:c r="I160"/>
+      <x:c r="J160"/>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="1" t="str">
@@ -4194,6 +4858,8 @@
       <x:c r="H161" s="1" t="str">
         <x:v>If speed drops, the set is done.</x:v>
       </x:c>
+      <x:c r="I161"/>
+      <x:c r="J161"/>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="1" t="str">
@@ -4218,6 +4884,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H162" s="1" t="str"/>
+      <x:c r="I162"/>
+      <x:c r="J162"/>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="1" t="str">
@@ -4242,6 +4910,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H163" s="1" t="str"/>
+      <x:c r="I163"/>
+      <x:c r="J163"/>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="1" t="str">
@@ -4266,6 +4936,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H164" s="1" t="str"/>
+      <x:c r="I164"/>
+      <x:c r="J164"/>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="1" t="str">
@@ -4290,6 +4962,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H165" s="1" t="str"/>
+      <x:c r="I165"/>
+      <x:c r="J165"/>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="1" t="str">
@@ -4314,6 +4988,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H166" s="1" t="str"/>
+      <x:c r="I166"/>
+      <x:c r="J166"/>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="1" t="str">
@@ -4338,6 +5014,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H167" s="1" t="str"/>
+      <x:c r="I167"/>
+      <x:c r="J167"/>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="1" t="str">
@@ -4362,6 +5040,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H168" s="1" t="str"/>
+      <x:c r="I168"/>
+      <x:c r="J168"/>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="1" t="str">
@@ -4388,6 +5068,8 @@
       <x:c r="H169" s="1" t="str">
         <x:v>Settle in, breathe steadily.</x:v>
       </x:c>
+      <x:c r="I169"/>
+      <x:c r="J169"/>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="1" t="str">
@@ -4412,6 +5094,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H170" s="1" t="str"/>
+      <x:c r="I170"/>
+      <x:c r="J170"/>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="1" t="str">
@@ -4436,6 +5120,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H171" s="1" t="str"/>
+      <x:c r="I171"/>
+      <x:c r="J171"/>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="1" t="str">
@@ -4460,6 +5146,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H172" s="1" t="str"/>
+      <x:c r="I172"/>
+      <x:c r="J172"/>
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="1" t="str">
@@ -4484,6 +5172,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H173" s="1" t="str"/>
+      <x:c r="I173"/>
+      <x:c r="J173"/>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="1" t="str">
@@ -4508,6 +5198,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H174" s="1" t="str"/>
+      <x:c r="I174"/>
+      <x:c r="J174"/>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="1" t="str">
@@ -4532,6 +5224,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H175" s="1" t="str"/>
+      <x:c r="I175"/>
+      <x:c r="J175"/>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="1" t="str">
@@ -4556,6 +5250,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H176" s="1" t="str"/>
+      <x:c r="I176"/>
+      <x:c r="J176"/>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="1" t="str">
@@ -4580,6 +5276,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H177" s="1" t="str"/>
+      <x:c r="I177"/>
+      <x:c r="J177"/>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="1" t="str">
@@ -4604,6 +5302,8 @@
         <x:v>Hit X number of calories every minute, the faster you do them the more rest you get.</x:v>
       </x:c>
       <x:c r="H178" s="1" t="str"/>
+      <x:c r="I178"/>
+      <x:c r="J178"/>
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="1" t="str">
@@ -4630,6 +5330,8 @@
       <x:c r="H179" s="1" t="str">
         <x:v>Controlled breathing throughout.</x:v>
       </x:c>
+      <x:c r="I179"/>
+      <x:c r="J179"/>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="1" t="str">
@@ -4654,6 +5356,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H180" s="1" t="str"/>
+      <x:c r="I180"/>
+      <x:c r="J180"/>
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="1" t="str">
@@ -4678,6 +5382,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H181" s="1" t="str"/>
+      <x:c r="I181"/>
+      <x:c r="J181"/>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="1" t="str">
@@ -4702,6 +5408,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H182" s="1" t="str"/>
+      <x:c r="I182"/>
+      <x:c r="J182"/>
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="1" t="str">
@@ -4726,6 +5434,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H183" s="1" t="str"/>
+      <x:c r="I183"/>
+      <x:c r="J183"/>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="1" t="str">
@@ -4750,6 +5460,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H184" s="1" t="str"/>
+      <x:c r="I184"/>
+      <x:c r="J184"/>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="1" t="str">
@@ -4776,6 +5488,8 @@
       <x:c r="H185" s="1" t="str">
         <x:v>Recover fully between sprints.</x:v>
       </x:c>
+      <x:c r="I185"/>
+      <x:c r="J185"/>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="1" t="str">
@@ -4802,6 +5516,8 @@
       <x:c r="H186" s="1" t="str">
         <x:v>Maintain power, recover completely.</x:v>
       </x:c>
+      <x:c r="I186"/>
+      <x:c r="J186"/>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="1" t="str">
@@ -4826,6 +5542,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H187" s="1" t="str"/>
+      <x:c r="I187"/>
+      <x:c r="J187"/>
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="1" t="str">
@@ -4850,6 +5568,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H188" s="1" t="str"/>
+      <x:c r="I188"/>
+      <x:c r="J188"/>
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="1" t="str">
@@ -4876,6 +5596,8 @@
       <x:c r="H189" s="1" t="str">
         <x:v>Move and loosen up.</x:v>
       </x:c>
+      <x:c r="I189"/>
+      <x:c r="J189"/>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="1" t="str">
@@ -4902,6 +5624,8 @@
       <x:c r="H190" s="1" t="str">
         <x:v>This is recovery, not training.</x:v>
       </x:c>
+      <x:c r="I190"/>
+      <x:c r="J190"/>
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="1" t="str">
@@ -4928,6 +5652,8 @@
       <x:c r="H191" s="1" t="str">
         <x:v>This is active recovery, not training.</x:v>
       </x:c>
+      <x:c r="I191"/>
+      <x:c r="J191"/>
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="1" t="str">
@@ -4954,6 +5680,8 @@
       <x:c r="H192" s="1" t="str">
         <x:v>Focus on form, not intensity.</x:v>
       </x:c>
+      <x:c r="I192"/>
+      <x:c r="J192"/>
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="1" t="str">
@@ -4978,6 +5706,8 @@
         <x:v>PENDING — Stage B</x:v>
       </x:c>
       <x:c r="H193" s="1" t="str"/>
+      <x:c r="I193"/>
+      <x:c r="J193"/>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="1" t="str">
@@ -5004,6 +5734,8 @@
       <x:c r="H194" s="1" t="str">
         <x:v>This is recovery, not intensity.</x:v>
       </x:c>
+      <x:c r="I194"/>
+      <x:c r="J194"/>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="1" t="str">
@@ -5028,6 +5760,8 @@
         <x:v>Try to run this at the same pace for the entire 2km</x:v>
       </x:c>
       <x:c r="H195" s="1" t="str"/>
+      <x:c r="I195"/>
+      <x:c r="J195"/>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="1"/>
@@ -5038,6 +5772,8 @@
       <x:c r="F196" s="1"/>
       <x:c r="G196" s="1"/>
       <x:c r="H196"/>
+      <x:c r="I196"/>
+      <x:c r="J196"/>
     </x:row>
     <x:row r="197">
       <x:c r="A197" t="str">
@@ -5062,6 +5798,8 @@
       <x:c r="H197" t="str">
         <x:v>Stop if reps get slow.</x:v>
       </x:c>
+      <x:c r="I197"/>
+      <x:c r="J197"/>
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="1" t="str">
@@ -5086,6 +5824,8 @@
         <x:v>Stand tall, jump and then bounce off the balls of your feet.</x:v>
       </x:c>
       <x:c r="H198" s="1" t="str"/>
+      <x:c r="I198"/>
+      <x:c r="J198"/>
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="1" t="str">
@@ -5110,6 +5850,8 @@
         <x:v>Jump off outside leg to the side, turn in air and land in a squat.</x:v>
       </x:c>
       <x:c r="H199" s="1" t="str"/>
+      <x:c r="I199"/>
+      <x:c r="J199"/>
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="1" t="str">
@@ -5134,6 +5876,8 @@
         <x:v>Start in kneeling position, jump onto feet, land in a squat.</x:v>
       </x:c>
       <x:c r="H200" s="1" t="str"/>
+      <x:c r="I200"/>
+      <x:c r="J200"/>
     </x:row>
     <x:row r="201">
       <x:c r="A201" s="1" t="str">
@@ -5160,6 +5904,12 @@
       <x:c r="H201" s="1" t="str">
         <x:v>Land soft and controlled.</x:v>
       </x:c>
+      <x:c r="I201" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J201" t="str">
+        <x:v>frontal, transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="202">
       <x:c r="A202" s="1" t="str">
@@ -5184,6 +5934,8 @@
       <x:c r="H202" s="1" t="str">
         <x:v>Stop when reps slow. Sore wrists? Elevate hands on box.</x:v>
       </x:c>
+      <x:c r="I202"/>
+      <x:c r="J202"/>
     </x:row>
     <x:row r="203">
       <x:c r="A203" s="1" t="str">
@@ -5210,6 +5962,8 @@
       <x:c r="H203" s="1" t="str">
         <x:v>Drive hard, fast lockout.</x:v>
       </x:c>
+      <x:c r="I203"/>
+      <x:c r="J203"/>
     </x:row>
     <x:row r="204">
       <x:c r="A204" s="1" t="str">
@@ -5234,6 +5988,8 @@
         <x:v>Wrap band around each side of bar, stand on band, get tight, explode up, control down.</x:v>
       </x:c>
       <x:c r="H204" s="1" t="str"/>
+      <x:c r="I204"/>
+      <x:c r="J204"/>
     </x:row>
     <x:row r="205">
       <x:c r="A205" s="1" t="str">
@@ -5260,6 +6016,10 @@
       <x:c r="H205" s="1" t="str">
         <x:v>Pause at the top.</x:v>
       </x:c>
+      <x:c r="I205" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J205" t="str"/>
     </x:row>
     <x:row r="206" ht="70" customHeight="1">
       <x:c r="A206" s="5" t="str">
@@ -5284,6 +6044,10 @@
         <x:v>Stand tall, lift one knee to 90 degrees, then straighten your leg.</x:v>
       </x:c>
       <x:c r="H206" s="5" t="str"/>
+      <x:c r="I206" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J206" t="str"/>
     </x:row>
     <x:row r="207" ht="70" customHeight="1">
       <x:c r="A207" s="5" t="str">
@@ -5310,6 +6074,8 @@
       <x:c r="H207" s="5" t="str">
         <x:v>Keep the chest open and hold.</x:v>
       </x:c>
+      <x:c r="I207"/>
+      <x:c r="J207"/>
     </x:row>
     <x:row r="208" ht="70" customHeight="1">
       <x:c r="A208" s="5" t="str">
@@ -5336,6 +6102,8 @@
       <x:c r="H208" s="5" t="str">
         <x:v>Don't round the spine.</x:v>
       </x:c>
+      <x:c r="I208"/>
+      <x:c r="J208"/>
     </x:row>
     <x:row r="209" ht="70" customHeight="1">
       <x:c r="A209" s="5" t="str">
@@ -5362,6 +6130,12 @@
       <x:c r="H209" s="5" t="str">
         <x:v>Keep the hips square and finish without arching the lower back.</x:v>
       </x:c>
+      <x:c r="I209" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J209" t="str">
+        <x:v>frontal, transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="210" ht="70" customHeight="1">
       <x:c r="A210" s="5" t="str">
@@ -5388,6 +6162,12 @@
       <x:c r="H210" s="5" t="str">
         <x:v>Keep the hips square and avoid hanging through the lower back.</x:v>
       </x:c>
+      <x:c r="I210" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J210" t="str">
+        <x:v>frontal, transverse</x:v>
+      </x:c>
     </x:row>
     <x:row r="211" ht="70" customHeight="1">
       <x:c r="A211" s="5" t="str">
@@ -5414,6 +6194,10 @@
       <x:c r="H211" s="5" t="str">
         <x:v>Keep knees, hips, and shoulders in one straight line.</x:v>
       </x:c>
+      <x:c r="I211" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J211" t="str"/>
     </x:row>
     <x:row r="212" ht="70" customHeight="1">
       <x:c r="A212" s="5" t="str">
@@ -5438,6 +6222,8 @@
         <x:v>Load the outside hip, rotate hard, and throw through the wall.</x:v>
       </x:c>
       <x:c r="H212" s="5" t="str"/>
+      <x:c r="I212"/>
+      <x:c r="J212"/>
     </x:row>
     <x:row r="213" ht="70" customHeight="1">
       <x:c r="A213" s="5" t="str">
@@ -5464,6 +6250,8 @@
       <x:c r="H213" s="5" t="str">
         <x:v>Finish athletically with the hips and knees softly bent.</x:v>
       </x:c>
+      <x:c r="I213"/>
+      <x:c r="J213"/>
     </x:row>
     <x:row r="214" ht="70" customHeight="1">
       <x:c r="A214" s="5" t="str">
@@ -5490,6 +6278,8 @@
       <x:c r="H214" s="5" t="str">
         <x:v>Reset before each explosive repetition.</x:v>
       </x:c>
+      <x:c r="I214"/>
+      <x:c r="J214"/>
     </x:row>
     <x:row r="215" ht="70" customHeight="1">
       <x:c r="A215" s="5" t="str">
@@ -5516,6 +6306,8 @@
       <x:c r="H215" s="5" t="str">
         <x:v>Push knees over toes and keep your torso tall.</x:v>
       </x:c>
+      <x:c r="I215"/>
+      <x:c r="J215"/>
     </x:row>
     <x:row r="216" ht="70" customHeight="1">
       <x:c r="A216" s="5" t="str">
@@ -5542,6 +6334,8 @@
       <x:c r="H216" s="5" t="str">
         <x:v>Sink your chest without arching through the lower back.</x:v>
       </x:c>
+      <x:c r="I216"/>
+      <x:c r="J216"/>
     </x:row>
     <x:row r="217" ht="90" customHeight="1">
       <x:c r="A217" s="5" t="str">
@@ -5568,6 +6362,8 @@
       <x:c r="H217" s="5" t="str">
         <x:v>Stop at a mild stretch behind the shoulder, never the front.</x:v>
       </x:c>
+      <x:c r="I217"/>
+      <x:c r="J217"/>
     </x:row>
     <x:row r="218">
       <x:c r="A218" s="5" t="str">
@@ -5594,6 +6390,8 @@
       <x:c r="H218" s="5" t="str">
         <x:v>Keep ribs tucked and avoid arching through the lower back.</x:v>
       </x:c>
+      <x:c r="I218"/>
+      <x:c r="J218"/>
     </x:row>
     <x:row r="219">
       <x:c r="A219" s="5" t="str">
@@ -5620,6 +6418,12 @@
       <x:c r="H219" s="5" t="str">
         <x:v>Lower under control until your elbows fully straighten.</x:v>
       </x:c>
+      <x:c r="I219" t="str">
+        <x:v>frontal</x:v>
+      </x:c>
+      <x:c r="J219" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="220" ht="72" customHeight="1">
       <x:c r="A220" s="5" t="str">
@@ -5646,6 +6450,12 @@
       <x:c r="H220" s="5" t="str">
         <x:v>Press away without letting your hips sag or shoulders shrug.</x:v>
       </x:c>
+      <x:c r="I220" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J220" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
     </x:row>
     <x:row r="221" ht="72" customHeight="1">
       <x:c r="A221" s="5" t="str">
@@ -5672,6 +6482,8 @@
       <x:c r="H221" s="5" t="str">
         <x:v>Land quietly, absorb through the hip, and hold your balance.</x:v>
       </x:c>
+      <x:c r="I221"/>
+      <x:c r="J221"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(programming): add shoulder rotation and COD cadence
Agent: movementplane
</commit_message>
<xml_diff>
--- a/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
+++ b/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Raa44463d67934fa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Rdc46445d78374de4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6485,6 +6485,36 @@
       <x:c r="I221"/>
       <x:c r="J221"/>
     </x:row>
+    <x:row r="222" ht="72" customHeight="1">
+      <x:c r="A222" s="5" t="str">
+        <x:v>Shoulder health</x:v>
+      </x:c>
+      <x:c r="B222" s="5" t="str">
+        <x:v>Banded 90/90 External Rotation</x:v>
+      </x:c>
+      <x:c r="C222" s="5" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="D222" s="5" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E222" s="5" t="str">
+        <x:v>everyone</x:v>
+      </x:c>
+      <x:c r="F222" s="5" t="str">
+        <x:v>Band resistance. 2 × 15–20 per arm with 20 seconds rest. Automatic in Shoulder health and upper-body warm-up slots; manual Add/Swap; not automatic in Primer. All phases and suitable at G-1 when pain-free.</x:v>
+      </x:c>
+      <x:c r="G222" s="5" t="str">
+        <x:v>Keep your elbow level with your shoulder and rotate your forearm upward.</x:v>
+      </x:c>
+      <x:c r="H222" s="5" t="str">
+        <x:v>Keep ribs down; avoid shrugging or forcing the range.</x:v>
+      </x:c>
+      <x:c r="I222" s="5" t="str">
+        <x:v>transverse</x:v>
+      </x:c>
+      <x:c r="J222" s="5"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add T-Bar Tib Raises and tib bar equipment
Agent: tibbar
</commit_message>
<xml_diff>
--- a/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
+++ b/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Rdc46445d78374de4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="Rc12a52bbaf874db2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -73,7 +73,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="7">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0"/>
@@ -81,6 +81,9 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -6515,6 +6518,36 @@
       </x:c>
       <x:c r="J222" s="5"/>
     </x:row>
+    <x:row r="223" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A223" s="5" t="str">
+        <x:v>Accessories lower</x:v>
+      </x:c>
+      <x:c r="B223" s="5" t="str">
+        <x:v>T-Bar Tib Raises</x:v>
+      </x:c>
+      <x:c r="C223" s="5" t="str">
+        <x:v>Calves</x:v>
+      </x:c>
+      <x:c r="D223" s="5" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E223" s="5" t="str">
+        <x:v>everyone</x:v>
+      </x:c>
+      <x:c r="F223" s="5" t="str">
+        <x:v>Tibialis anterior (shin). Requires a tib bar and compatible plates. Uses the Tib Raises dose: 2 × 15–20 reps with 30 seconds rest. Begin empty or light, record total external load, and retain full ankle range. Automatic progression from Tib Raises when available; manual Add/Swap. All phases; familiar light loading is suitable at G-1.</x:v>
+      </x:c>
+      <x:c r="G223" s="5" t="str">
+        <x:v>Pull your toes toward your shins through the full range.</x:v>
+      </x:c>
+      <x:c r="H223" s="5" t="str">
+        <x:v>Keep knees still, pause at the top, and lower under control.</x:v>
+      </x:c>
+      <x:c r="I223" s="6" t="str">
+        <x:v>sagittal</x:v>
+      </x:c>
+      <x:c r="J223" s="6"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Fix final weekly composition guards
Agent: fourconfirmed
</commit_message>
<xml_diff>
--- a/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
+++ b/docs/EXERCISE_MASTER_SHEET_2026-07-28.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="R1592cfa65e4f47f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Master" sheetId="1" r:id="R1436b8cd7dc548a0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -383,6 +383,7 @@
     <x:col min="8" max="8" width="60" customWidth="1"/>
     <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -402,6 +403,9 @@
       <x:c r="J1" s="5" t="str">
         <x:v>Blank = unanswered</x:v>
       </x:c>
+      <x:c r="K1" s="5" t="str">
+        <x:v>ACCESSORY AFFINITY — 2026-09-02</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="1" t="str">
@@ -420,6 +424,9 @@
       <x:c r="J2" s="5" t="str">
         <x:v>multiplanar · not_applicable</x:v>
       </x:c>
+      <x:c r="K2" s="5" t="str">
+        <x:v>push · pull · both</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
@@ -434,6 +441,7 @@
       <x:c r="H3"/>
       <x:c r="I3"/>
       <x:c r="J3"/>
+      <x:c r="K3" s="5"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="1" t="str">
@@ -448,6 +456,7 @@
       <x:c r="H4"/>
       <x:c r="I4"/>
       <x:c r="J4"/>
+      <x:c r="K4" s="5"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
@@ -462,6 +471,7 @@
       <x:c r="H5"/>
       <x:c r="I5"/>
       <x:c r="J5"/>
+      <x:c r="K5" s="5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="2" t="str">
@@ -494,6 +504,9 @@
       <x:c r="J6" s="5" t="str">
         <x:v>Secondary Plane(s)</x:v>
       </x:c>
+      <x:c r="K6" s="5" t="str">
+        <x:v>Accessory Affinity</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1" t="str">
@@ -522,6 +535,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J7" t="str"/>
+      <x:c r="K7" s="5"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="str">
@@ -552,6 +566,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J8" t="str"/>
+      <x:c r="K8" s="5"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="str">
@@ -580,6 +595,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J9" t="str"/>
+      <x:c r="K9" s="5"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="1" t="str">
@@ -606,6 +622,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J10" t="str"/>
+      <x:c r="K10" s="5"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="str">
@@ -636,6 +653,7 @@
       <x:c r="J11" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K11" s="5"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1" t="str">
@@ -666,6 +684,7 @@
       <x:c r="J12" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K12" s="5"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1" t="str">
@@ -696,6 +715,7 @@
       <x:c r="J13" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K13" s="5"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1" t="str">
@@ -726,6 +746,7 @@
       <x:c r="J14" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K14" s="5"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1" t="str">
@@ -754,6 +775,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J15" t="str"/>
+      <x:c r="K15" s="5"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1" t="str">
@@ -782,6 +804,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J16" t="str"/>
+      <x:c r="K16" s="5"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="1" t="str">
@@ -810,6 +833,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J17" t="str"/>
+      <x:c r="K17" s="5"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="1" t="str">
@@ -840,6 +864,7 @@
       <x:c r="J18" t="str">
         <x:v>frontal, transverse</x:v>
       </x:c>
+      <x:c r="K18" s="5"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="1" t="str">
@@ -864,6 +889,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J19" t="str"/>
+      <x:c r="K19" s="5"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="1" t="str">
@@ -894,6 +920,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J20" t="str"/>
+      <x:c r="K20" s="5"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="1" t="str">
@@ -922,6 +949,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J21" t="str"/>
+      <x:c r="K21" s="5"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="1" t="str">
@@ -952,6 +980,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J22" t="str"/>
+      <x:c r="K22" s="5"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="1" t="str">
@@ -982,6 +1011,7 @@
       <x:c r="J23" t="str">
         <x:v>frontal, transverse</x:v>
       </x:c>
+      <x:c r="K23" s="5"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="1" t="str">
@@ -1010,6 +1040,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J24" t="str"/>
+      <x:c r="K24" s="5"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="1" t="str">
@@ -1038,6 +1069,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J25" t="str"/>
+      <x:c r="K25" s="5"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="1" t="str">
@@ -1064,6 +1096,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J26" t="str"/>
+      <x:c r="K26" s="5"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="1" t="str">
@@ -1092,6 +1125,7 @@
         <x:v>transverse</x:v>
       </x:c>
       <x:c r="J27" t="str"/>
+      <x:c r="K27" s="5"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="1" t="str">
@@ -1122,6 +1156,7 @@
       <x:c r="J28" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K28" s="5"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="1" t="str">
@@ -1152,6 +1187,7 @@
       <x:c r="J29" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K29" s="5"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="1" t="str">
@@ -1180,6 +1216,7 @@
         <x:v>transverse</x:v>
       </x:c>
       <x:c r="J30" t="str"/>
+      <x:c r="K30" s="5"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="1" t="str">
@@ -1210,6 +1247,7 @@
       <x:c r="J31" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K31" s="5"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="1" t="str">
@@ -1240,6 +1278,7 @@
       <x:c r="J32" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K32" s="5"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="1" t="str">
@@ -1268,6 +1307,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J33" t="str"/>
+      <x:c r="K33" s="5"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="1" t="str">
@@ -1298,6 +1338,7 @@
         <x:v>transverse</x:v>
       </x:c>
       <x:c r="J34" t="str"/>
+      <x:c r="K34" s="5"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="1" t="str">
@@ -1328,6 +1369,7 @@
         <x:v>transverse</x:v>
       </x:c>
       <x:c r="J35" t="str"/>
+      <x:c r="K35" s="5"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="1" t="str">
@@ -1358,6 +1400,7 @@
       <x:c r="J36" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K36" s="5"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="1" t="str">
@@ -1390,6 +1433,7 @@
       <x:c r="J37" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K37" s="5"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="1" t="str">
@@ -1420,6 +1464,7 @@
       <x:c r="J38" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K38" s="5"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="1" t="str">
@@ -1450,6 +1495,7 @@
       <x:c r="J39" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K39" s="5"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="1" t="str">
@@ -1480,6 +1526,7 @@
       <x:c r="J40" t="str">
         <x:v>transverse</x:v>
       </x:c>
+      <x:c r="K40" s="5"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="1" t="str">
@@ -1510,6 +1557,7 @@
       <x:c r="J41" t="str">
         <x:v>transverse</x:v>
       </x:c>
+      <x:c r="K41" s="5"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="1" t="str">
@@ -1542,6 +1590,7 @@
       <x:c r="J42" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K42" s="5"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="1" t="str">
@@ -1572,6 +1621,7 @@
       <x:c r="J43" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K43" s="5"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="1" t="str">
@@ -1604,6 +1654,7 @@
       <x:c r="J44" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K44" s="5"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="1" t="str">
@@ -1634,6 +1685,7 @@
       <x:c r="J45" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K45" s="5"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="1" t="str">
@@ -1664,6 +1716,7 @@
       <x:c r="J46" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K46" s="5"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="1" t="str">
@@ -1694,6 +1747,9 @@
       <x:c r="J47" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K47" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="1" t="str">
@@ -1722,6 +1778,9 @@
         <x:v>transverse</x:v>
       </x:c>
       <x:c r="J48" t="str"/>
+      <x:c r="K48" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="1" t="str">
@@ -1750,6 +1809,9 @@
         <x:v>transverse</x:v>
       </x:c>
       <x:c r="J49" t="str"/>
+      <x:c r="K49" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="1" t="str">
@@ -1780,6 +1842,7 @@
       <x:c r="J50" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K50" s="5"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="1" t="str">
@@ -1810,6 +1873,7 @@
       <x:c r="J51" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K51" s="5"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="1" t="str">
@@ -1840,6 +1904,7 @@
       <x:c r="J52" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K52" s="5"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="1" t="str">
@@ -1868,6 +1933,7 @@
       <x:c r="J53" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K53" s="5"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="1" t="str">
@@ -1900,6 +1966,7 @@
       <x:c r="J54" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K54" s="5"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="1" t="str">
@@ -1928,6 +1995,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J55" t="str"/>
+      <x:c r="K55" s="5"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="1" t="str">
@@ -1956,6 +2024,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J56" t="str"/>
+      <x:c r="K56" s="5"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="1" t="str">
@@ -1984,6 +2053,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J57" t="str"/>
+      <x:c r="K57" s="5"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="1" t="str">
@@ -2016,6 +2086,7 @@
       <x:c r="J58" t="str">
         <x:v>transverse</x:v>
       </x:c>
+      <x:c r="K58" s="5"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="1" t="str">
@@ -2048,6 +2119,7 @@
       <x:c r="J59" t="str">
         <x:v>frontal, transverse</x:v>
       </x:c>
+      <x:c r="K59" s="5"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="1" t="str">
@@ -2078,6 +2150,7 @@
       <x:c r="J60" t="str">
         <x:v>frontal, transverse</x:v>
       </x:c>
+      <x:c r="K60" s="5"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="1" t="str">
@@ -2108,6 +2181,7 @@
       <x:c r="J61" t="str">
         <x:v>transverse</x:v>
       </x:c>
+      <x:c r="K61" s="5"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="1" t="str">
@@ -2138,6 +2212,7 @@
       <x:c r="J62" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K62" s="5"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="1" t="str">
@@ -2168,6 +2243,7 @@
       <x:c r="J63" t="str">
         <x:v>frontal, transverse</x:v>
       </x:c>
+      <x:c r="K63" s="5"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="1" t="str">
@@ -2196,6 +2272,9 @@
         <x:v>frontal</x:v>
       </x:c>
       <x:c r="J64" t="str"/>
+      <x:c r="K64" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="1" t="str">
@@ -2226,6 +2305,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J65" t="str"/>
+      <x:c r="K65" s="5" t="str">
+        <x:v>push</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="1" t="str">
@@ -2254,6 +2336,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J66" t="str"/>
+      <x:c r="K66" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="1" t="str">
@@ -2282,6 +2367,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J67" t="str"/>
+      <x:c r="K67" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="1" t="str">
@@ -2310,6 +2398,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J68" t="str"/>
+      <x:c r="K68" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="1" t="str">
@@ -2338,6 +2429,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J69" t="str"/>
+      <x:c r="K69" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="1" t="str">
@@ -2366,6 +2460,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J70" t="str"/>
+      <x:c r="K70" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="1" t="str">
@@ -2396,6 +2493,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J71" t="str"/>
+      <x:c r="K71" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="1" t="str">
@@ -2424,6 +2524,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J72" t="str"/>
+      <x:c r="K72" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="1" t="str">
@@ -2452,6 +2555,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J73" t="str"/>
+      <x:c r="K73" s="5" t="str">
+        <x:v>push</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="1" t="str">
@@ -2480,6 +2586,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J74" t="str"/>
+      <x:c r="K74" s="5" t="str">
+        <x:v>push</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="1" t="str">
@@ -2508,6 +2617,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J75" t="str"/>
+      <x:c r="K75" s="5" t="str">
+        <x:v>push</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="1" t="str">
@@ -2538,6 +2650,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J76" t="str"/>
+      <x:c r="K76" s="5" t="str">
+        <x:v>push</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="1" t="str">
@@ -2566,6 +2681,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J77" t="str"/>
+      <x:c r="K77" s="5" t="str">
+        <x:v>push</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="1" t="str">
@@ -2594,6 +2712,9 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J78" t="str"/>
+      <x:c r="K78" s="5" t="str">
+        <x:v>push</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="1" t="str">
@@ -2622,6 +2743,9 @@
         <x:v>frontal</x:v>
       </x:c>
       <x:c r="J79" t="str"/>
+      <x:c r="K79" s="5" t="str">
+        <x:v>push</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="1" t="str">
@@ -2652,6 +2776,9 @@
       <x:c r="J80" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K80" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="1" t="str">
@@ -2680,6 +2807,9 @@
         <x:v>frontal</x:v>
       </x:c>
       <x:c r="J81" t="str"/>
+      <x:c r="K81" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="1" t="str">
@@ -2710,6 +2840,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J82" t="str"/>
+      <x:c r="K82" s="5"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="1" t="str">
@@ -2736,6 +2867,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J83" t="str"/>
+      <x:c r="K83" s="5"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="1" t="str">
@@ -2762,6 +2894,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J84" t="str"/>
+      <x:c r="K84" s="5"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="1" t="str">
@@ -2790,6 +2923,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J85" t="str"/>
+      <x:c r="K85" s="5"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="1" t="str">
@@ -2820,6 +2954,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J86" t="str"/>
+      <x:c r="K86" s="5"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="1" t="str">
@@ -2848,6 +2983,7 @@
       <x:c r="J87" t="str">
         <x:v>frontal, transverse</x:v>
       </x:c>
+      <x:c r="K87" s="5"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="1" t="str">
@@ -2876,6 +3012,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J88" t="str"/>
+      <x:c r="K88" s="5"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="1" t="str">
@@ -2908,6 +3045,7 @@
       <x:c r="J89" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K89" s="5"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" t="str">
@@ -2938,6 +3076,9 @@
       <x:c r="J90" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K90" s="5" t="str">
+        <x:v>pull</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="1" t="str">
@@ -2968,6 +3109,7 @@
       <x:c r="J91" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K91" s="5"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="1" t="str">
@@ -2998,6 +3140,7 @@
       <x:c r="J92" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K92" s="5"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="1" t="str">
@@ -3028,6 +3171,7 @@
       <x:c r="J93" t="str">
         <x:v>transverse</x:v>
       </x:c>
+      <x:c r="K93" s="5"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="1" t="str">
@@ -3058,6 +3202,7 @@
       <x:c r="J94" t="str">
         <x:v>transverse</x:v>
       </x:c>
+      <x:c r="K94" s="5"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="1" t="str">
@@ -3086,6 +3231,7 @@
         <x:v>frontal</x:v>
       </x:c>
       <x:c r="J95" t="str"/>
+      <x:c r="K95" s="5"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="1" t="str">
@@ -3116,6 +3262,7 @@
       <x:c r="J96" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K96" s="5"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="1" t="str">
@@ -3146,6 +3293,7 @@
       <x:c r="J97" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K97" s="5"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="1" t="str">
@@ -3176,6 +3324,7 @@
       <x:c r="J98" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K98" s="5"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="1" t="str">
@@ -3204,6 +3353,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J99" t="str"/>
+      <x:c r="K99" s="5"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="1" t="str">
@@ -3230,6 +3380,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J100" t="str"/>
+      <x:c r="K100" s="5"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="1" t="str">
@@ -3258,6 +3409,7 @@
       <x:c r="J101" t="str">
         <x:v>frontal, transverse</x:v>
       </x:c>
+      <x:c r="K101" s="5"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="1" t="str">
@@ -3284,6 +3436,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J102" t="str"/>
+      <x:c r="K102" s="5"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="1" t="str">
@@ -3312,6 +3465,7 @@
       <x:c r="J103" t="str">
         <x:v>frontal</x:v>
       </x:c>
+      <x:c r="K103" s="5"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="1" t="str">
@@ -3340,6 +3494,7 @@
       <x:c r="J104" t="str">
         <x:v>transverse</x:v>
       </x:c>
+      <x:c r="K104" s="5"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="1" t="str">
@@ -3368,6 +3523,7 @@
         <x:v>transverse</x:v>
       </x:c>
       <x:c r="J105" t="str"/>
+      <x:c r="K105" s="5"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="1" t="str">
@@ -3398,6 +3554,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J106" t="str"/>
+      <x:c r="K106" s="5"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="1" t="str">
@@ -3426,6 +3583,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J107" t="str"/>
+      <x:c r="K107" s="5"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="1" t="str">
@@ -3454,6 +3612,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J108" t="str"/>
+      <x:c r="K108" s="5"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="1" t="str">
@@ -3482,6 +3641,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J109" t="str"/>
+      <x:c r="K109" s="5"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="1" t="str">
@@ -3512,6 +3672,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J110" t="str"/>
+      <x:c r="K110" s="5"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="1" t="str">
@@ -3540,6 +3701,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J111" t="str"/>
+      <x:c r="K111" s="5"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="1" t="str">
@@ -3572,6 +3734,7 @@
       <x:c r="J112" t="str">
         <x:v>transverse</x:v>
       </x:c>
+      <x:c r="K112" s="5"/>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="1" t="str">
@@ -3602,6 +3765,7 @@
       <x:c r="J113" t="str">
         <x:v>transverse</x:v>
       </x:c>
+      <x:c r="K113" s="5"/>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="1" t="str">
@@ -3630,6 +3794,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J114" t="str"/>
+      <x:c r="K114" s="5"/>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="1" t="str">
@@ -3656,6 +3821,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J115" t="str"/>
+      <x:c r="K115" s="5"/>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="1" t="str">
@@ -3682,6 +3848,7 @@
         <x:v>multiplanar</x:v>
       </x:c>
       <x:c r="J116" t="str"/>
+      <x:c r="K116" s="5"/>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="1" t="str">
@@ -3710,6 +3877,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J117" t="str"/>
+      <x:c r="K117" s="5"/>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="1" t="str">
@@ -3738,6 +3906,7 @@
       <x:c r="J118" t="str">
         <x:v>transverse</x:v>
       </x:c>
+      <x:c r="K118" s="5"/>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="1" t="str">
@@ -3768,6 +3937,7 @@
       <x:c r="J119" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K119" s="5"/>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="1" t="str">
@@ -3798,6 +3968,7 @@
       <x:c r="J120" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K120" s="5"/>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="1" t="str">
@@ -3824,6 +3995,7 @@
       </x:c>
       <x:c r="I121"/>
       <x:c r="J121"/>
+      <x:c r="K121" s="5"/>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="1" t="str">
@@ -3852,6 +4024,7 @@
       </x:c>
       <x:c r="I122"/>
       <x:c r="J122"/>
+      <x:c r="K122" s="5"/>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="1" t="str">
@@ -3878,6 +4051,7 @@
       </x:c>
       <x:c r="I123"/>
       <x:c r="J123"/>
+      <x:c r="K123" s="5"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="1" t="str">
@@ -3906,6 +4080,7 @@
       <x:c r="J124" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K124" s="5"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="1" t="str">
@@ -3934,6 +4109,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J125" t="str"/>
+      <x:c r="K125" s="5"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="1" t="str">
@@ -3960,6 +4136,7 @@
       </x:c>
       <x:c r="I126"/>
       <x:c r="J126"/>
+      <x:c r="K126" s="5"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="1" t="str">
@@ -3986,6 +4163,7 @@
       </x:c>
       <x:c r="I127"/>
       <x:c r="J127"/>
+      <x:c r="K127" s="5"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="1" t="str">
@@ -4012,6 +4190,7 @@
       </x:c>
       <x:c r="I128"/>
       <x:c r="J128"/>
+      <x:c r="K128" s="5"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="1" t="str">
@@ -4038,6 +4217,7 @@
       </x:c>
       <x:c r="I129"/>
       <x:c r="J129"/>
+      <x:c r="K129" s="5"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="1" t="str">
@@ -4064,6 +4244,7 @@
       </x:c>
       <x:c r="I130"/>
       <x:c r="J130"/>
+      <x:c r="K130" s="5"/>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="1" t="str">
@@ -4090,6 +4271,7 @@
       </x:c>
       <x:c r="I131"/>
       <x:c r="J131"/>
+      <x:c r="K131" s="5"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="1" t="str">
@@ -4116,6 +4298,7 @@
       </x:c>
       <x:c r="I132"/>
       <x:c r="J132"/>
+      <x:c r="K132" s="5"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="1" t="str">
@@ -4142,6 +4325,7 @@
       </x:c>
       <x:c r="I133"/>
       <x:c r="J133"/>
+      <x:c r="K133" s="5"/>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="1" t="str">
@@ -4168,6 +4352,7 @@
       </x:c>
       <x:c r="I134"/>
       <x:c r="J134"/>
+      <x:c r="K134" s="5"/>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="1" t="str">
@@ -4194,6 +4379,7 @@
       </x:c>
       <x:c r="I135"/>
       <x:c r="J135"/>
+      <x:c r="K135" s="5"/>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="1" t="str">
@@ -4220,6 +4406,7 @@
       </x:c>
       <x:c r="I136"/>
       <x:c r="J136"/>
+      <x:c r="K136" s="5"/>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="1" t="str">
@@ -4246,6 +4433,7 @@
       </x:c>
       <x:c r="I137"/>
       <x:c r="J137"/>
+      <x:c r="K137" s="5"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="1" t="str">
@@ -4272,6 +4460,7 @@
       </x:c>
       <x:c r="I138"/>
       <x:c r="J138"/>
+      <x:c r="K138" s="5"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="1" t="str">
@@ -4298,6 +4487,7 @@
       </x:c>
       <x:c r="I139"/>
       <x:c r="J139"/>
+      <x:c r="K139" s="5"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="1" t="str">
@@ -4324,6 +4514,7 @@
       </x:c>
       <x:c r="I140"/>
       <x:c r="J140"/>
+      <x:c r="K140" s="5"/>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="1" t="str">
@@ -4350,6 +4541,7 @@
       </x:c>
       <x:c r="I141"/>
       <x:c r="J141"/>
+      <x:c r="K141" s="5"/>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="1" t="str">
@@ -4376,6 +4568,7 @@
       </x:c>
       <x:c r="I142"/>
       <x:c r="J142"/>
+      <x:c r="K142" s="5"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="1" t="str">
@@ -4404,6 +4597,7 @@
       </x:c>
       <x:c r="I143"/>
       <x:c r="J143"/>
+      <x:c r="K143" s="5"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="1" t="str">
@@ -4430,6 +4624,7 @@
       </x:c>
       <x:c r="I144"/>
       <x:c r="J144"/>
+      <x:c r="K144" s="5"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="1" t="str">
@@ -4456,6 +4651,7 @@
       <x:c r="H145" s="1" t="str"/>
       <x:c r="I145"/>
       <x:c r="J145"/>
+      <x:c r="K145" s="5"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="1" t="str">
@@ -4482,6 +4678,7 @@
       <x:c r="H146" s="1" t="str"/>
       <x:c r="I146"/>
       <x:c r="J146"/>
+      <x:c r="K146" s="5"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="1" t="str">
@@ -4506,6 +4703,7 @@
       <x:c r="H147" s="1" t="str"/>
       <x:c r="I147"/>
       <x:c r="J147"/>
+      <x:c r="K147" s="5"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="1" t="str">
@@ -4530,6 +4728,7 @@
       <x:c r="H148" s="1" t="str"/>
       <x:c r="I148"/>
       <x:c r="J148"/>
+      <x:c r="K148" s="5"/>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="1" t="str">
@@ -4554,6 +4753,7 @@
       <x:c r="H149" s="1" t="str"/>
       <x:c r="I149"/>
       <x:c r="J149"/>
+      <x:c r="K149" s="5"/>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="1" t="str">
@@ -4578,6 +4778,7 @@
       <x:c r="H150" s="1" t="str"/>
       <x:c r="I150"/>
       <x:c r="J150"/>
+      <x:c r="K150" s="5"/>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="1" t="str">
@@ -4602,6 +4803,7 @@
       <x:c r="H151" s="1" t="str"/>
       <x:c r="I151"/>
       <x:c r="J151"/>
+      <x:c r="K151" s="5"/>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="1" t="str">
@@ -4628,6 +4830,7 @@
       </x:c>
       <x:c r="I152"/>
       <x:c r="J152"/>
+      <x:c r="K152" s="5"/>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="1" t="str">
@@ -4654,6 +4857,7 @@
       </x:c>
       <x:c r="I153"/>
       <x:c r="J153"/>
+      <x:c r="K153" s="5"/>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="1" t="str">
@@ -4680,6 +4884,7 @@
       </x:c>
       <x:c r="I154"/>
       <x:c r="J154"/>
+      <x:c r="K154" s="5"/>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="1" t="str">
@@ -4706,6 +4911,7 @@
       </x:c>
       <x:c r="I155"/>
       <x:c r="J155"/>
+      <x:c r="K155" s="5"/>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="1" t="str">
@@ -4732,6 +4938,7 @@
       </x:c>
       <x:c r="I156"/>
       <x:c r="J156"/>
+      <x:c r="K156" s="5"/>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="1" t="str">
@@ -4758,6 +4965,7 @@
       </x:c>
       <x:c r="I157"/>
       <x:c r="J157"/>
+      <x:c r="K157" s="5"/>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="1" t="str">
@@ -4784,6 +4992,7 @@
       </x:c>
       <x:c r="I158"/>
       <x:c r="J158"/>
+      <x:c r="K158" s="5"/>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="1" t="str">
@@ -4812,6 +5021,7 @@
       </x:c>
       <x:c r="I159"/>
       <x:c r="J159"/>
+      <x:c r="K159" s="5"/>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="1" t="str">
@@ -4840,6 +5050,7 @@
       </x:c>
       <x:c r="I160"/>
       <x:c r="J160"/>
+      <x:c r="K160" s="5"/>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="1" t="str">
@@ -4868,6 +5079,7 @@
       </x:c>
       <x:c r="I161"/>
       <x:c r="J161"/>
+      <x:c r="K161" s="5"/>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="1" t="str">
@@ -4894,6 +5106,7 @@
       <x:c r="H162" s="1" t="str"/>
       <x:c r="I162"/>
       <x:c r="J162"/>
+      <x:c r="K162" s="5"/>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="1" t="str">
@@ -4920,6 +5133,7 @@
       <x:c r="H163" s="1" t="str"/>
       <x:c r="I163"/>
       <x:c r="J163"/>
+      <x:c r="K163" s="5"/>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="1" t="str">
@@ -4946,6 +5160,7 @@
       <x:c r="H164" s="1" t="str"/>
       <x:c r="I164"/>
       <x:c r="J164"/>
+      <x:c r="K164" s="5"/>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="1" t="str">
@@ -4972,6 +5187,7 @@
       <x:c r="H165" s="1" t="str"/>
       <x:c r="I165"/>
       <x:c r="J165"/>
+      <x:c r="K165" s="5"/>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="1" t="str">
@@ -4998,6 +5214,7 @@
       <x:c r="H166" s="1" t="str"/>
       <x:c r="I166"/>
       <x:c r="J166"/>
+      <x:c r="K166" s="5"/>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="1" t="str">
@@ -5024,6 +5241,7 @@
       <x:c r="H167" s="1" t="str"/>
       <x:c r="I167"/>
       <x:c r="J167"/>
+      <x:c r="K167" s="5"/>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="1" t="str">
@@ -5050,6 +5268,7 @@
       <x:c r="H168" s="1" t="str"/>
       <x:c r="I168"/>
       <x:c r="J168"/>
+      <x:c r="K168" s="5"/>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="1" t="str">
@@ -5078,6 +5297,7 @@
       </x:c>
       <x:c r="I169"/>
       <x:c r="J169"/>
+      <x:c r="K169" s="5"/>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="1" t="str">
@@ -5104,6 +5324,7 @@
       <x:c r="H170" s="1" t="str"/>
       <x:c r="I170"/>
       <x:c r="J170"/>
+      <x:c r="K170" s="5"/>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="1" t="str">
@@ -5130,6 +5351,7 @@
       <x:c r="H171" s="1" t="str"/>
       <x:c r="I171"/>
       <x:c r="J171"/>
+      <x:c r="K171" s="5"/>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="1" t="str">
@@ -5156,6 +5378,7 @@
       <x:c r="H172" s="1" t="str"/>
       <x:c r="I172"/>
       <x:c r="J172"/>
+      <x:c r="K172" s="5"/>
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="1" t="str">
@@ -5182,6 +5405,7 @@
       <x:c r="H173" s="1" t="str"/>
       <x:c r="I173"/>
       <x:c r="J173"/>
+      <x:c r="K173" s="5"/>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="1" t="str">
@@ -5208,6 +5432,7 @@
       <x:c r="H174" s="1" t="str"/>
       <x:c r="I174"/>
       <x:c r="J174"/>
+      <x:c r="K174" s="5"/>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="1" t="str">
@@ -5234,6 +5459,7 @@
       <x:c r="H175" s="1" t="str"/>
       <x:c r="I175"/>
       <x:c r="J175"/>
+      <x:c r="K175" s="5"/>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="1" t="str">
@@ -5260,6 +5486,7 @@
       <x:c r="H176" s="1" t="str"/>
       <x:c r="I176"/>
       <x:c r="J176"/>
+      <x:c r="K176" s="5"/>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="1" t="str">
@@ -5286,6 +5513,7 @@
       <x:c r="H177" s="1" t="str"/>
       <x:c r="I177"/>
       <x:c r="J177"/>
+      <x:c r="K177" s="5"/>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="1" t="str">
@@ -5312,6 +5540,7 @@
       <x:c r="H178" s="1" t="str"/>
       <x:c r="I178"/>
       <x:c r="J178"/>
+      <x:c r="K178" s="5"/>
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="1" t="str">
@@ -5340,6 +5569,7 @@
       </x:c>
       <x:c r="I179"/>
       <x:c r="J179"/>
+      <x:c r="K179" s="5"/>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="1" t="str">
@@ -5366,6 +5596,7 @@
       <x:c r="H180" s="1" t="str"/>
       <x:c r="I180"/>
       <x:c r="J180"/>
+      <x:c r="K180" s="5"/>
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="1" t="str">
@@ -5392,6 +5623,7 @@
       <x:c r="H181" s="1" t="str"/>
       <x:c r="I181"/>
       <x:c r="J181"/>
+      <x:c r="K181" s="5"/>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="1" t="str">
@@ -5418,6 +5650,7 @@
       <x:c r="H182" s="1" t="str"/>
       <x:c r="I182"/>
       <x:c r="J182"/>
+      <x:c r="K182" s="5"/>
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="1" t="str">
@@ -5444,6 +5677,7 @@
       <x:c r="H183" s="1" t="str"/>
       <x:c r="I183"/>
       <x:c r="J183"/>
+      <x:c r="K183" s="5"/>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="1" t="str">
@@ -5470,6 +5704,7 @@
       <x:c r="H184" s="1" t="str"/>
       <x:c r="I184"/>
       <x:c r="J184"/>
+      <x:c r="K184" s="5"/>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="1" t="str">
@@ -5498,6 +5733,7 @@
       </x:c>
       <x:c r="I185"/>
       <x:c r="J185"/>
+      <x:c r="K185" s="5"/>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="1" t="str">
@@ -5526,6 +5762,7 @@
       </x:c>
       <x:c r="I186"/>
       <x:c r="J186"/>
+      <x:c r="K186" s="5"/>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="1" t="str">
@@ -5552,6 +5789,7 @@
       <x:c r="H187" s="1" t="str"/>
       <x:c r="I187"/>
       <x:c r="J187"/>
+      <x:c r="K187" s="5"/>
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="1" t="str">
@@ -5578,6 +5816,7 @@
       <x:c r="H188" s="1" t="str"/>
       <x:c r="I188"/>
       <x:c r="J188"/>
+      <x:c r="K188" s="5"/>
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="1" t="str">
@@ -5606,6 +5845,7 @@
       </x:c>
       <x:c r="I189"/>
       <x:c r="J189"/>
+      <x:c r="K189" s="5"/>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="1" t="str">
@@ -5634,6 +5874,7 @@
       </x:c>
       <x:c r="I190"/>
       <x:c r="J190"/>
+      <x:c r="K190" s="5"/>
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="1" t="str">
@@ -5662,6 +5903,7 @@
       </x:c>
       <x:c r="I191"/>
       <x:c r="J191"/>
+      <x:c r="K191" s="5"/>
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="1" t="str">
@@ -5690,6 +5932,7 @@
       </x:c>
       <x:c r="I192"/>
       <x:c r="J192"/>
+      <x:c r="K192" s="5"/>
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="1" t="str">
@@ -5716,6 +5959,7 @@
       <x:c r="H193" s="1" t="str"/>
       <x:c r="I193"/>
       <x:c r="J193"/>
+      <x:c r="K193" s="5"/>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="1" t="str">
@@ -5744,6 +5988,7 @@
       </x:c>
       <x:c r="I194"/>
       <x:c r="J194"/>
+      <x:c r="K194" s="5"/>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="1" t="str">
@@ -5770,6 +6015,7 @@
       <x:c r="H195" s="1" t="str"/>
       <x:c r="I195"/>
       <x:c r="J195"/>
+      <x:c r="K195" s="5"/>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="1"/>
@@ -5782,6 +6028,7 @@
       <x:c r="H196"/>
       <x:c r="I196"/>
       <x:c r="J196"/>
+      <x:c r="K196" s="5"/>
     </x:row>
     <x:row r="197">
       <x:c r="A197" t="str">
@@ -5810,6 +6057,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J197" t="str"/>
+      <x:c r="K197" s="5"/>
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="1" t="str">
@@ -5838,6 +6086,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J198" t="str"/>
+      <x:c r="K198" s="5"/>
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="1" t="str">
@@ -5868,6 +6117,7 @@
       <x:c r="J199" t="str">
         <x:v>transverse</x:v>
       </x:c>
+      <x:c r="K199" s="5"/>
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="1" t="str">
@@ -5896,6 +6146,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J200" t="str"/>
+      <x:c r="K200" s="5"/>
     </x:row>
     <x:row r="201">
       <x:c r="A201" s="1" t="str">
@@ -5928,6 +6179,7 @@
       <x:c r="J201" t="str">
         <x:v>frontal, transverse</x:v>
       </x:c>
+      <x:c r="K201" s="5"/>
     </x:row>
     <x:row r="202">
       <x:c r="A202" s="1" t="str">
@@ -5958,6 +6210,7 @@
       <x:c r="J202" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K202" s="5"/>
     </x:row>
     <x:row r="203">
       <x:c r="A203" s="1" t="str">
@@ -5986,6 +6239,7 @@
       </x:c>
       <x:c r="I203"/>
       <x:c r="J203"/>
+      <x:c r="K203" s="5"/>
     </x:row>
     <x:row r="204">
       <x:c r="A204" s="1" t="str">
@@ -6012,6 +6266,7 @@
       <x:c r="H204" s="1" t="str"/>
       <x:c r="I204"/>
       <x:c r="J204"/>
+      <x:c r="K204" s="5"/>
     </x:row>
     <x:row r="205">
       <x:c r="A205" s="1" t="str">
@@ -6042,6 +6297,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J205" t="str"/>
+      <x:c r="K205" s="5"/>
     </x:row>
     <x:row r="206" ht="70" customHeight="1">
       <x:c r="A206" s="5" t="str">
@@ -6070,6 +6326,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J206" t="str"/>
+      <x:c r="K206" s="5"/>
     </x:row>
     <x:row r="207" ht="70" customHeight="1">
       <x:c r="A207" s="5" t="str">
@@ -6098,6 +6355,7 @@
       </x:c>
       <x:c r="I207"/>
       <x:c r="J207"/>
+      <x:c r="K207" s="5"/>
     </x:row>
     <x:row r="208" ht="70" customHeight="1">
       <x:c r="A208" s="5" t="str">
@@ -6126,6 +6384,7 @@
       </x:c>
       <x:c r="I208"/>
       <x:c r="J208"/>
+      <x:c r="K208" s="5"/>
     </x:row>
     <x:row r="209" ht="70" customHeight="1">
       <x:c r="A209" s="5" t="str">
@@ -6158,6 +6417,7 @@
       <x:c r="J209" t="str">
         <x:v>frontal, transverse</x:v>
       </x:c>
+      <x:c r="K209" s="5"/>
     </x:row>
     <x:row r="210" ht="70" customHeight="1">
       <x:c r="A210" s="5" t="str">
@@ -6190,6 +6450,7 @@
       <x:c r="J210" t="str">
         <x:v>frontal, transverse</x:v>
       </x:c>
+      <x:c r="K210" s="5"/>
     </x:row>
     <x:row r="211" ht="70" customHeight="1">
       <x:c r="A211" s="5" t="str">
@@ -6220,6 +6481,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J211" t="str"/>
+      <x:c r="K211" s="5"/>
     </x:row>
     <x:row r="212" ht="70" customHeight="1">
       <x:c r="A212" s="5" t="str">
@@ -6250,6 +6512,7 @@
       <x:c r="J212" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K212" s="5"/>
     </x:row>
     <x:row r="213" ht="70" customHeight="1">
       <x:c r="A213" s="5" t="str">
@@ -6280,6 +6543,7 @@
         <x:v>sagittal</x:v>
       </x:c>
       <x:c r="J213" t="str"/>
+      <x:c r="K213" s="5"/>
     </x:row>
     <x:row r="214" ht="70" customHeight="1">
       <x:c r="A214" s="5" t="str">
@@ -6312,6 +6576,7 @@
       <x:c r="J214" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K214" s="5"/>
     </x:row>
     <x:row r="215" ht="70" customHeight="1">
       <x:c r="A215" s="5" t="str">
@@ -6340,6 +6605,7 @@
       </x:c>
       <x:c r="I215"/>
       <x:c r="J215"/>
+      <x:c r="K215" s="5"/>
     </x:row>
     <x:row r="216" ht="70" customHeight="1">
       <x:c r="A216" s="5" t="str">
@@ -6368,6 +6634,7 @@
       </x:c>
       <x:c r="I216"/>
       <x:c r="J216"/>
+      <x:c r="K216" s="5"/>
     </x:row>
     <x:row r="217" ht="90" customHeight="1">
       <x:c r="A217" s="5" t="str">
@@ -6396,6 +6663,7 @@
       </x:c>
       <x:c r="I217"/>
       <x:c r="J217"/>
+      <x:c r="K217" s="5"/>
     </x:row>
     <x:row r="218">
       <x:c r="A218" s="5" t="str">
@@ -6424,6 +6692,7 @@
       </x:c>
       <x:c r="I218"/>
       <x:c r="J218"/>
+      <x:c r="K218" s="5"/>
     </x:row>
     <x:row r="219">
       <x:c r="A219" s="5" t="str">
@@ -6456,6 +6725,7 @@
       <x:c r="J219" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K219" s="5"/>
     </x:row>
     <x:row r="220" ht="72" customHeight="1">
       <x:c r="A220" s="5" t="str">
@@ -6488,6 +6758,7 @@
       <x:c r="J220" t="str">
         <x:v>sagittal</x:v>
       </x:c>
+      <x:c r="K220" s="5"/>
     </x:row>
     <x:row r="221" ht="72" customHeight="1">
       <x:c r="A221" s="5" t="str">
@@ -6520,6 +6791,7 @@
       <x:c r="J221" t="str">
         <x:v>frontal, transverse</x:v>
       </x:c>
+      <x:c r="K221" s="5"/>
     </x:row>
     <x:row r="222" ht="72" customHeight="1">
       <x:c r="A222" s="5" t="str">
@@ -6550,6 +6822,7 @@
         <x:v>transverse</x:v>
       </x:c>
       <x:c r="J222" s="5"/>
+      <x:c r="K222" s="5"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>